<commit_message>
Updated HRV_grids_kan10 model - 2026-08-26 14:52
</commit_message>
<xml_diff>
--- a/VerveStacks_HRV_grids_kan10/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_HRV_grids_kan10/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_HRV_grids_kan10\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D27C4A2C-5DBB-410F-B9C8-F1AE1D1A775C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0BC6102C-5CD0-4AC1-9A82-A90B2CE98D76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1261,49 +1261,49 @@
     <t>grid_node</t>
   </si>
   <si>
-    <t>p_w113757307-220_HRV</t>
-  </si>
-  <si>
-    <t>p_w162022271-220_HRV</t>
-  </si>
-  <si>
-    <t>p_w163860997-400_HRV</t>
-  </si>
-  <si>
-    <t>p_w170366194-220_HRV</t>
-  </si>
-  <si>
-    <t>p_w210745193-220_HRV</t>
-  </si>
-  <si>
-    <t>p_w273326173-220_HRV</t>
-  </si>
-  <si>
-    <t>p_w43337263-220_HRV</t>
-  </si>
-  <si>
-    <t>p_w43337263-400_HRV</t>
-  </si>
-  <si>
-    <t>p_w89817617-220_HRV</t>
-  </si>
-  <si>
-    <t>p_w89817617-400_HRV</t>
-  </si>
-  <si>
-    <t>p_w89818719-400_HRV</t>
-  </si>
-  <si>
-    <t>p_w89819945-220_HRV</t>
-  </si>
-  <si>
-    <t>p_w89820062-400_HRV</t>
-  </si>
-  <si>
-    <t>p_w89823918-400_HRV</t>
-  </si>
-  <si>
-    <t>p_w96704507-220_HRV</t>
+    <t>p_Vinkovci_HRV</t>
+  </si>
+  <si>
+    <t>p_Sibenik_HRV</t>
+  </si>
+  <si>
+    <t>p_Knin_HRV</t>
+  </si>
+  <si>
+    <t>p_Sisak_HRV</t>
+  </si>
+  <si>
+    <t>p_Pula_HRV</t>
+  </si>
+  <si>
+    <t>p_Ogulin_HRV</t>
+  </si>
+  <si>
+    <t>p_Split_HRV</t>
+  </si>
+  <si>
+    <t>p_KastelStari_HRV</t>
+  </si>
+  <si>
+    <t>p_Viskovo_HRV</t>
+  </si>
+  <si>
+    <t>p_Rijeka_HRV</t>
+  </si>
+  <si>
+    <t>p_VelikaGorica_HRV</t>
+  </si>
+  <si>
+    <t>p_Sesvete_HRV</t>
+  </si>
+  <si>
+    <t>p_Zagreb_HRV</t>
+  </si>
+  <si>
+    <t>p_Osijek_HRV</t>
+  </si>
+  <si>
+    <t>p_Kutina_HRV</t>
   </si>
   <si>
     <t>rez_spv_HRV_001</t>
@@ -1399,49 +1399,49 @@
     <t>region_com</t>
   </si>
   <si>
-    <t>e_w113757307-220_HRV</t>
-  </si>
-  <si>
-    <t>e_w162022271-220_HRV</t>
-  </si>
-  <si>
-    <t>e_w163860997-400_HRV</t>
-  </si>
-  <si>
-    <t>e_w170366194-220_HRV</t>
-  </si>
-  <si>
-    <t>e_w210745193-220_HRV</t>
-  </si>
-  <si>
-    <t>e_w273326173-220_HRV</t>
-  </si>
-  <si>
-    <t>e_w43337263-220_HRV</t>
-  </si>
-  <si>
-    <t>e_w43337263-400_HRV</t>
-  </si>
-  <si>
-    <t>e_w89817617-220_HRV</t>
-  </si>
-  <si>
-    <t>e_w89817617-400_HRV</t>
-  </si>
-  <si>
-    <t>e_w89818719-400_HRV</t>
-  </si>
-  <si>
-    <t>e_w89819945-220_HRV</t>
-  </si>
-  <si>
-    <t>e_w89820062-400_HRV</t>
-  </si>
-  <si>
-    <t>e_w89823918-400_HRV</t>
-  </si>
-  <si>
-    <t>e_w96704507-220_HRV</t>
+    <t>e_Vinkovci_HRV</t>
+  </si>
+  <si>
+    <t>e_Sibenik_HRV</t>
+  </si>
+  <si>
+    <t>e_Knin_HRV</t>
+  </si>
+  <si>
+    <t>e_Sisak_HRV</t>
+  </si>
+  <si>
+    <t>e_Pula_HRV</t>
+  </si>
+  <si>
+    <t>e_Ogulin_HRV</t>
+  </si>
+  <si>
+    <t>e_Split_HRV</t>
+  </si>
+  <si>
+    <t>e_KastelStari_HRV</t>
+  </si>
+  <si>
+    <t>e_Viskovo_HRV</t>
+  </si>
+  <si>
+    <t>e_Rijeka_HRV</t>
+  </si>
+  <si>
+    <t>e_VelikaGorica_HRV</t>
+  </si>
+  <si>
+    <t>e_Sesvete_HRV</t>
+  </si>
+  <si>
+    <t>e_Zagreb_HRV</t>
+  </si>
+  <si>
+    <t>e_Osijek_HRV</t>
+  </si>
+  <si>
+    <t>e_Kutina_HRV</t>
   </si>
   <si>
     <t>elc_spv_HRV_001</t>
@@ -1537,49 +1537,49 @@
     <t>lng</t>
   </si>
   <si>
-    <t>HRV-e_w113757307-220_HRV</t>
-  </si>
-  <si>
-    <t>HRV-e_w162022271-220_HRV</t>
-  </si>
-  <si>
-    <t>HRV-e_w163860997-400_HRV</t>
-  </si>
-  <si>
-    <t>HRV-e_w170366194-220_HRV</t>
-  </si>
-  <si>
-    <t>HRV-e_w210745193-220_HRV</t>
-  </si>
-  <si>
-    <t>HRV-e_w273326173-220_HRV</t>
-  </si>
-  <si>
-    <t>HRV-e_w43337263-220_HRV</t>
-  </si>
-  <si>
-    <t>HRV-e_w43337263-400_HRV</t>
-  </si>
-  <si>
-    <t>HRV-e_w89817617-220_HRV</t>
-  </si>
-  <si>
-    <t>HRV-e_w89817617-400_HRV</t>
-  </si>
-  <si>
-    <t>HRV-e_w89818719-400_HRV</t>
-  </si>
-  <si>
-    <t>HRV-e_w89819945-220_HRV</t>
-  </si>
-  <si>
-    <t>HRV-e_w89820062-400_HRV</t>
-  </si>
-  <si>
-    <t>HRV-e_w89823918-400_HRV</t>
-  </si>
-  <si>
-    <t>HRV-e_w96704507-220_HRV</t>
+    <t>HRV-e_Vinkovci_HRV</t>
+  </si>
+  <si>
+    <t>HRV-e_Sibenik_HRV</t>
+  </si>
+  <si>
+    <t>HRV-e_Knin_HRV</t>
+  </si>
+  <si>
+    <t>HRV-e_Sisak_HRV</t>
+  </si>
+  <si>
+    <t>HRV-e_Pula_HRV</t>
+  </si>
+  <si>
+    <t>HRV-e_Ogulin_HRV</t>
+  </si>
+  <si>
+    <t>HRV-e_Split_HRV</t>
+  </si>
+  <si>
+    <t>HRV-e_KastelStari_HRV</t>
+  </si>
+  <si>
+    <t>HRV-e_Viskovo_HRV</t>
+  </si>
+  <si>
+    <t>HRV-e_Rijeka_HRV</t>
+  </si>
+  <si>
+    <t>HRV-e_VelikaGorica_HRV</t>
+  </si>
+  <si>
+    <t>HRV-e_Sesvete_HRV</t>
+  </si>
+  <si>
+    <t>HRV-e_Zagreb_HRV</t>
+  </si>
+  <si>
+    <t>HRV-e_Osijek_HRV</t>
+  </si>
+  <si>
+    <t>HRV-e_Kutina_HRV</t>
   </si>
   <si>
     <t>HRV-elc_spv_HRV_001</t>
@@ -22464,7 +22464,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93CFF3C2-C02A-4E47-85A4-C2BC47B6796F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC7567E7-E11D-4D00-B408-C308454F7196}">
   <dimension ref="B9:H53"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -23362,7 +23362,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46A32C73-0920-4789-BD7A-A8C83E821EC1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{23069963-69FE-425B-A4E1-8C0EA618D319}">
   <dimension ref="B9:L53"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated HRV_grids_kan10 model - 2026-08-26 19:40
</commit_message>
<xml_diff>
--- a/VerveStacks_HRV_grids_kan10/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_HRV_grids_kan10/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_HRV_grids_kan10\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EAD3044B-C014-4703-BA7A-F88FCD6698E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E3D01803-E5E5-4643-BC0C-E1E0BC4362D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="8" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2607,7 +2607,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6EBAD231-B145-443A-B9BC-05ACA40FE98F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F903696-05EB-428B-A102-DDC1A4807837}">
   <dimension ref="B9:L53"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -25748,7 +25748,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF552863-B344-4566-9A1D-19309532F921}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{209D560C-BF42-4D8D-ACD6-9B1A2B13C8DD}">
   <dimension ref="B9:H53"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated HRV_grids_kan10 model - 2026-08-26 21:40
</commit_message>
<xml_diff>
--- a/VerveStacks_HRV_grids_kan10/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_HRV_grids_kan10/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_HRV_grids_kan10\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E3D01803-E5E5-4643-BC0C-E1E0BC4362D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4000B349-900A-4394-BD11-4D0A42D3F148}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="8" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2607,7 +2607,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F903696-05EB-428B-A102-DDC1A4807837}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B1FAD15-D88D-46FA-8DDC-2E25F9265204}">
   <dimension ref="B9:L53"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -25748,7 +25748,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{209D560C-BF42-4D8D-ACD6-9B1A2B13C8DD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0DE4908D-2988-4109-BF0F-AFAF04A74C42}">
   <dimension ref="B9:H53"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated HRV_grids_kan10 model - 2026-08-27 01:13
</commit_message>
<xml_diff>
--- a/VerveStacks_HRV_grids_kan10/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_HRV_grids_kan10/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_HRV_grids_kan10\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4000B349-900A-4394-BD11-4D0A42D3F148}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{47576E11-B6CF-4204-B00E-549CD0699BA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="8" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2607,7 +2607,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B1FAD15-D88D-46FA-8DDC-2E25F9265204}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1614E75E-962B-48D0-A72F-E08B47BAB23F}">
   <dimension ref="B9:L53"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -25748,7 +25748,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0DE4908D-2988-4109-BF0F-AFAF04A74C42}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14D1024C-CB50-4338-8309-6783BE3B28B4}">
   <dimension ref="B9:H53"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated HRV_grids_kan10 model - 2026-08-27 10:17
</commit_message>
<xml_diff>
--- a/VerveStacks_HRV_grids_kan10/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_HRV_grids_kan10/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_HRV_grids_kan10\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{47576E11-B6CF-4204-B00E-549CD0699BA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{06CEF92E-74AF-48B8-8439-E10CEA7165C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="8" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -83,7 +83,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5479" uniqueCount="532">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5836" uniqueCount="644">
   <si>
     <t>Unit</t>
   </si>
@@ -1321,6 +1321,54 @@
     <t>p_Kutina_HRV</t>
   </si>
   <si>
+    <t>s_ogci10893_HRV</t>
+  </si>
+  <si>
+    <t>s_ogci10894_HRV</t>
+  </si>
+  <si>
+    <t>s_ogci10895_HRV</t>
+  </si>
+  <si>
+    <t>s_ogci10896_HRV</t>
+  </si>
+  <si>
+    <t>s_ogci10897_HRV</t>
+  </si>
+  <si>
+    <t>s_ogci10898_HRV</t>
+  </si>
+  <si>
+    <t>s_ogci10899_HRV</t>
+  </si>
+  <si>
+    <t>s_ogci10900_HRV</t>
+  </si>
+  <si>
+    <t>s_ogci10901_HRV</t>
+  </si>
+  <si>
+    <t>s_ogci10902_HRV</t>
+  </si>
+  <si>
+    <t>s_ogci10903_HRV</t>
+  </si>
+  <si>
+    <t>s_ogci10904_HRV</t>
+  </si>
+  <si>
+    <t>s_ogci10906_HRV</t>
+  </si>
+  <si>
+    <t>s_ogci10907_HRV</t>
+  </si>
+  <si>
+    <t>s_ogci11249_HRV</t>
+  </si>
+  <si>
+    <t>s_ogci11250_HRV</t>
+  </si>
+  <si>
     <t>rez_spv_HRV_001</t>
   </si>
   <si>
@@ -1405,12 +1453,48 @@
     <t>rez_won_HRV_013</t>
   </si>
   <si>
+    <t>rez_wof_HRV_001</t>
+  </si>
+  <si>
+    <t>rez_wof_HRV_002</t>
+  </si>
+  <si>
+    <t>rez_wof_HRV_003</t>
+  </si>
+  <si>
+    <t>rez_wof_HRV_004</t>
+  </si>
+  <si>
+    <t>rez_wof_HRV_005</t>
+  </si>
+  <si>
+    <t>rez_wof_HRV_006</t>
+  </si>
+  <si>
+    <t>rez_wof_HRV_007</t>
+  </si>
+  <si>
+    <t>rez_wof_HRV_008</t>
+  </si>
+  <si>
+    <t>rez_wof_HRV_009</t>
+  </si>
+  <si>
+    <t>rez_wof_HRV_010</t>
+  </si>
+  <si>
+    <t>rez_wof_HRV_011</t>
+  </si>
+  <si>
     <t>admin_1</t>
   </si>
   <si>
     <t>Hrvatska</t>
   </si>
   <si>
+    <t>Unknown</t>
+  </si>
+  <si>
     <t>region_com</t>
   </si>
   <si>
@@ -1543,6 +1627,132 @@
     <t>elc_won_HRV_013</t>
   </si>
   <si>
+    <t>elc_wof_HRV_001</t>
+  </si>
+  <si>
+    <t>elc_wof_HRV_002</t>
+  </si>
+  <si>
+    <t>elc_wof_HRV_003</t>
+  </si>
+  <si>
+    <t>elc_wof_HRV_004</t>
+  </si>
+  <si>
+    <t>elc_wof_HRV_005</t>
+  </si>
+  <si>
+    <t>elc_wof_HRV_006</t>
+  </si>
+  <si>
+    <t>elc_wof_HRV_007</t>
+  </si>
+  <si>
+    <t>elc_wof_HRV_008</t>
+  </si>
+  <si>
+    <t>elc_wof_HRV_009</t>
+  </si>
+  <si>
+    <t>elc_wof_HRV_010</t>
+  </si>
+  <si>
+    <t>elc_wof_HRV_011</t>
+  </si>
+  <si>
+    <t>co2_Vinkovci_HRV</t>
+  </si>
+  <si>
+    <t>co2_Sibenik_HRV</t>
+  </si>
+  <si>
+    <t>co2_Knin_HRV</t>
+  </si>
+  <si>
+    <t>co2_Sisak_HRV</t>
+  </si>
+  <si>
+    <t>co2_Pula_HRV</t>
+  </si>
+  <si>
+    <t>co2_Ogulin_HRV</t>
+  </si>
+  <si>
+    <t>co2_Split_HRV</t>
+  </si>
+  <si>
+    <t>co2_KastelStari_HRV</t>
+  </si>
+  <si>
+    <t>co2_Viskovo_HRV</t>
+  </si>
+  <si>
+    <t>co2_Rijeka_HRV</t>
+  </si>
+  <si>
+    <t>co2_VelikaGorica_HRV</t>
+  </si>
+  <si>
+    <t>co2_Sesvete_HRV</t>
+  </si>
+  <si>
+    <t>co2_Zagreb_HRV</t>
+  </si>
+  <si>
+    <t>co2_Osijek_HRV</t>
+  </si>
+  <si>
+    <t>co2_Kutina_HRV</t>
+  </si>
+  <si>
+    <t>co2s_ogci10893_HRV</t>
+  </si>
+  <si>
+    <t>co2s_ogci10894_HRV</t>
+  </si>
+  <si>
+    <t>co2s_ogci10895_HRV</t>
+  </si>
+  <si>
+    <t>co2s_ogci10896_HRV</t>
+  </si>
+  <si>
+    <t>co2s_ogci10897_HRV</t>
+  </si>
+  <si>
+    <t>co2s_ogci10898_HRV</t>
+  </si>
+  <si>
+    <t>co2s_ogci10899_HRV</t>
+  </si>
+  <si>
+    <t>co2s_ogci10900_HRV</t>
+  </si>
+  <si>
+    <t>co2s_ogci10901_HRV</t>
+  </si>
+  <si>
+    <t>co2s_ogci10902_HRV</t>
+  </si>
+  <si>
+    <t>co2s_ogci10903_HRV</t>
+  </si>
+  <si>
+    <t>co2s_ogci10904_HRV</t>
+  </si>
+  <si>
+    <t>co2s_ogci10906_HRV</t>
+  </si>
+  <si>
+    <t>co2s_ogci10907_HRV</t>
+  </si>
+  <si>
+    <t>co2s_ogci11249_HRV</t>
+  </si>
+  <si>
+    <t>co2s_ogci11250_HRV</t>
+  </si>
+  <si>
     <t>~geolocation</t>
   </si>
   <si>
@@ -1679,6 +1889,132 @@
   </si>
   <si>
     <t>HRV-elc_won_HRV_013</t>
+  </si>
+  <si>
+    <t>HRV-elc_wof_HRV_001</t>
+  </si>
+  <si>
+    <t>HRV-elc_wof_HRV_002</t>
+  </si>
+  <si>
+    <t>HRV-elc_wof_HRV_003</t>
+  </si>
+  <si>
+    <t>HRV-elc_wof_HRV_004</t>
+  </si>
+  <si>
+    <t>HRV-elc_wof_HRV_005</t>
+  </si>
+  <si>
+    <t>HRV-elc_wof_HRV_006</t>
+  </si>
+  <si>
+    <t>HRV-elc_wof_HRV_007</t>
+  </si>
+  <si>
+    <t>HRV-elc_wof_HRV_008</t>
+  </si>
+  <si>
+    <t>HRV-elc_wof_HRV_009</t>
+  </si>
+  <si>
+    <t>HRV-elc_wof_HRV_010</t>
+  </si>
+  <si>
+    <t>HRV-elc_wof_HRV_011</t>
+  </si>
+  <si>
+    <t>HRV-co2_Vinkovci_HRV</t>
+  </si>
+  <si>
+    <t>HRV-co2_Sibenik_HRV</t>
+  </si>
+  <si>
+    <t>HRV-co2_Knin_HRV</t>
+  </si>
+  <si>
+    <t>HRV-co2_Sisak_HRV</t>
+  </si>
+  <si>
+    <t>HRV-co2_Pula_HRV</t>
+  </si>
+  <si>
+    <t>HRV-co2_Ogulin_HRV</t>
+  </si>
+  <si>
+    <t>HRV-co2_Split_HRV</t>
+  </si>
+  <si>
+    <t>HRV-co2_KastelStari_HRV</t>
+  </si>
+  <si>
+    <t>HRV-co2_Viskovo_HRV</t>
+  </si>
+  <si>
+    <t>HRV-co2_Rijeka_HRV</t>
+  </si>
+  <si>
+    <t>HRV-co2_VelikaGorica_HRV</t>
+  </si>
+  <si>
+    <t>HRV-co2_Sesvete_HRV</t>
+  </si>
+  <si>
+    <t>HRV-co2_Zagreb_HRV</t>
+  </si>
+  <si>
+    <t>HRV-co2_Osijek_HRV</t>
+  </si>
+  <si>
+    <t>HRV-co2_Kutina_HRV</t>
+  </si>
+  <si>
+    <t>HRV-co2s_ogci10893_HRV</t>
+  </si>
+  <si>
+    <t>HRV-co2s_ogci10894_HRV</t>
+  </si>
+  <si>
+    <t>HRV-co2s_ogci10895_HRV</t>
+  </si>
+  <si>
+    <t>HRV-co2s_ogci10896_HRV</t>
+  </si>
+  <si>
+    <t>HRV-co2s_ogci10897_HRV</t>
+  </si>
+  <si>
+    <t>HRV-co2s_ogci10898_HRV</t>
+  </si>
+  <si>
+    <t>HRV-co2s_ogci10899_HRV</t>
+  </si>
+  <si>
+    <t>HRV-co2s_ogci10900_HRV</t>
+  </si>
+  <si>
+    <t>HRV-co2s_ogci10901_HRV</t>
+  </si>
+  <si>
+    <t>HRV-co2s_ogci10902_HRV</t>
+  </si>
+  <si>
+    <t>HRV-co2s_ogci10903_HRV</t>
+  </si>
+  <si>
+    <t>HRV-co2s_ogci10904_HRV</t>
+  </si>
+  <si>
+    <t>HRV-co2s_ogci10906_HRV</t>
+  </si>
+  <si>
+    <t>HRV-co2s_ogci10907_HRV</t>
+  </si>
+  <si>
+    <t>HRV-co2s_ogci11249_HRV</t>
+  </si>
+  <si>
+    <t>HRV-co2s_ogci11250_HRV</t>
   </si>
 </sst>
 </file>
@@ -2607,8 +2943,8 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1614E75E-962B-48D0-A72F-E08B47BAB23F}">
-  <dimension ref="B9:L53"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42CFE670-67E0-4416-855C-F02BC7EDF6DC}">
+  <dimension ref="B9:L95"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
     <row r="9" spans="2:12">
@@ -2665,19 +3001,19 @@
         <v>397</v>
       </c>
       <c r="G11" t="s">
-        <v>440</v>
+        <v>467</v>
       </c>
       <c r="H11" t="s">
-        <v>441</v>
+        <v>468</v>
       </c>
       <c r="J11" t="s">
-        <v>442</v>
+        <v>470</v>
       </c>
       <c r="K11" t="s">
-        <v>443</v>
+        <v>471</v>
       </c>
       <c r="L11" t="s">
-        <v>443</v>
+        <v>471</v>
       </c>
     </row>
     <row r="12" spans="2:12">
@@ -2694,19 +3030,19 @@
         <v>398</v>
       </c>
       <c r="G12" t="s">
-        <v>440</v>
+        <v>467</v>
       </c>
       <c r="H12" t="s">
-        <v>441</v>
+        <v>468</v>
       </c>
       <c r="J12" t="s">
-        <v>442</v>
+        <v>470</v>
       </c>
       <c r="K12" t="s">
-        <v>444</v>
+        <v>472</v>
       </c>
       <c r="L12" t="s">
-        <v>444</v>
+        <v>472</v>
       </c>
     </row>
     <row r="13" spans="2:12">
@@ -2723,19 +3059,19 @@
         <v>399</v>
       </c>
       <c r="G13" t="s">
-        <v>440</v>
+        <v>467</v>
       </c>
       <c r="H13" t="s">
-        <v>441</v>
+        <v>468</v>
       </c>
       <c r="J13" t="s">
-        <v>442</v>
+        <v>470</v>
       </c>
       <c r="K13" t="s">
-        <v>445</v>
+        <v>473</v>
       </c>
       <c r="L13" t="s">
-        <v>445</v>
+        <v>473</v>
       </c>
     </row>
     <row r="14" spans="2:12">
@@ -2752,19 +3088,19 @@
         <v>400</v>
       </c>
       <c r="G14" t="s">
-        <v>440</v>
+        <v>467</v>
       </c>
       <c r="H14" t="s">
-        <v>441</v>
+        <v>468</v>
       </c>
       <c r="J14" t="s">
-        <v>442</v>
+        <v>470</v>
       </c>
       <c r="K14" t="s">
-        <v>446</v>
+        <v>474</v>
       </c>
       <c r="L14" t="s">
-        <v>446</v>
+        <v>474</v>
       </c>
     </row>
     <row r="15" spans="2:12">
@@ -2781,19 +3117,19 @@
         <v>401</v>
       </c>
       <c r="G15" t="s">
-        <v>440</v>
+        <v>467</v>
       </c>
       <c r="H15" t="s">
-        <v>441</v>
+        <v>468</v>
       </c>
       <c r="J15" t="s">
-        <v>442</v>
+        <v>470</v>
       </c>
       <c r="K15" t="s">
-        <v>447</v>
+        <v>475</v>
       </c>
       <c r="L15" t="s">
-        <v>447</v>
+        <v>475</v>
       </c>
     </row>
     <row r="16" spans="2:12">
@@ -2810,19 +3146,19 @@
         <v>402</v>
       </c>
       <c r="G16" t="s">
-        <v>440</v>
+        <v>467</v>
       </c>
       <c r="H16" t="s">
-        <v>441</v>
+        <v>468</v>
       </c>
       <c r="J16" t="s">
-        <v>442</v>
+        <v>470</v>
       </c>
       <c r="K16" t="s">
-        <v>448</v>
+        <v>476</v>
       </c>
       <c r="L16" t="s">
-        <v>448</v>
+        <v>476</v>
       </c>
     </row>
     <row r="17" spans="2:12">
@@ -2839,19 +3175,19 @@
         <v>403</v>
       </c>
       <c r="G17" t="s">
-        <v>440</v>
+        <v>467</v>
       </c>
       <c r="H17" t="s">
-        <v>441</v>
+        <v>468</v>
       </c>
       <c r="J17" t="s">
-        <v>442</v>
+        <v>470</v>
       </c>
       <c r="K17" t="s">
-        <v>449</v>
+        <v>477</v>
       </c>
       <c r="L17" t="s">
-        <v>449</v>
+        <v>477</v>
       </c>
     </row>
     <row r="18" spans="2:12">
@@ -2868,19 +3204,19 @@
         <v>404</v>
       </c>
       <c r="G18" t="s">
-        <v>440</v>
+        <v>467</v>
       </c>
       <c r="H18" t="s">
-        <v>441</v>
+        <v>468</v>
       </c>
       <c r="J18" t="s">
-        <v>442</v>
+        <v>470</v>
       </c>
       <c r="K18" t="s">
-        <v>450</v>
+        <v>478</v>
       </c>
       <c r="L18" t="s">
-        <v>450</v>
+        <v>478</v>
       </c>
     </row>
     <row r="19" spans="2:12">
@@ -2897,19 +3233,19 @@
         <v>405</v>
       </c>
       <c r="G19" t="s">
-        <v>440</v>
+        <v>467</v>
       </c>
       <c r="H19" t="s">
-        <v>441</v>
+        <v>468</v>
       </c>
       <c r="J19" t="s">
-        <v>442</v>
+        <v>470</v>
       </c>
       <c r="K19" t="s">
-        <v>451</v>
+        <v>479</v>
       </c>
       <c r="L19" t="s">
-        <v>451</v>
+        <v>479</v>
       </c>
     </row>
     <row r="20" spans="2:12">
@@ -2926,19 +3262,19 @@
         <v>406</v>
       </c>
       <c r="G20" t="s">
-        <v>440</v>
+        <v>467</v>
       </c>
       <c r="H20" t="s">
-        <v>441</v>
+        <v>468</v>
       </c>
       <c r="J20" t="s">
-        <v>442</v>
+        <v>470</v>
       </c>
       <c r="K20" t="s">
-        <v>452</v>
+        <v>480</v>
       </c>
       <c r="L20" t="s">
-        <v>452</v>
+        <v>480</v>
       </c>
     </row>
     <row r="21" spans="2:12">
@@ -2955,19 +3291,19 @@
         <v>407</v>
       </c>
       <c r="G21" t="s">
-        <v>440</v>
+        <v>467</v>
       </c>
       <c r="H21" t="s">
-        <v>441</v>
+        <v>468</v>
       </c>
       <c r="J21" t="s">
-        <v>442</v>
+        <v>470</v>
       </c>
       <c r="K21" t="s">
-        <v>453</v>
+        <v>481</v>
       </c>
       <c r="L21" t="s">
-        <v>453</v>
+        <v>481</v>
       </c>
     </row>
     <row r="22" spans="2:12">
@@ -2984,19 +3320,19 @@
         <v>408</v>
       </c>
       <c r="G22" t="s">
-        <v>440</v>
+        <v>467</v>
       </c>
       <c r="H22" t="s">
-        <v>441</v>
+        <v>468</v>
       </c>
       <c r="J22" t="s">
-        <v>442</v>
+        <v>470</v>
       </c>
       <c r="K22" t="s">
-        <v>454</v>
+        <v>482</v>
       </c>
       <c r="L22" t="s">
-        <v>454</v>
+        <v>482</v>
       </c>
     </row>
     <row r="23" spans="2:12">
@@ -3013,19 +3349,19 @@
         <v>409</v>
       </c>
       <c r="G23" t="s">
-        <v>440</v>
+        <v>467</v>
       </c>
       <c r="H23" t="s">
-        <v>441</v>
+        <v>468</v>
       </c>
       <c r="J23" t="s">
-        <v>442</v>
+        <v>470</v>
       </c>
       <c r="K23" t="s">
-        <v>455</v>
+        <v>483</v>
       </c>
       <c r="L23" t="s">
-        <v>455</v>
+        <v>483</v>
       </c>
     </row>
     <row r="24" spans="2:12">
@@ -3042,19 +3378,19 @@
         <v>410</v>
       </c>
       <c r="G24" t="s">
-        <v>440</v>
+        <v>467</v>
       </c>
       <c r="H24" t="s">
-        <v>441</v>
+        <v>468</v>
       </c>
       <c r="J24" t="s">
-        <v>442</v>
+        <v>470</v>
       </c>
       <c r="K24" t="s">
-        <v>456</v>
+        <v>484</v>
       </c>
       <c r="L24" t="s">
-        <v>456</v>
+        <v>484</v>
       </c>
     </row>
     <row r="25" spans="2:12">
@@ -3071,19 +3407,19 @@
         <v>411</v>
       </c>
       <c r="G25" t="s">
-        <v>440</v>
+        <v>467</v>
       </c>
       <c r="H25" t="s">
-        <v>441</v>
+        <v>468</v>
       </c>
       <c r="J25" t="s">
-        <v>442</v>
+        <v>470</v>
       </c>
       <c r="K25" t="s">
-        <v>457</v>
+        <v>485</v>
       </c>
       <c r="L25" t="s">
-        <v>457</v>
+        <v>485</v>
       </c>
     </row>
     <row r="26" spans="2:12">
@@ -3097,22 +3433,22 @@
         <v>412</v>
       </c>
       <c r="F26" t="s">
-        <v>412</v>
+        <v>428</v>
       </c>
       <c r="G26" t="s">
-        <v>440</v>
+        <v>467</v>
       </c>
       <c r="H26" t="s">
-        <v>441</v>
+        <v>468</v>
       </c>
       <c r="J26" t="s">
-        <v>442</v>
+        <v>470</v>
       </c>
       <c r="K26" t="s">
-        <v>458</v>
+        <v>486</v>
       </c>
       <c r="L26" t="s">
-        <v>458</v>
+        <v>486</v>
       </c>
     </row>
     <row r="27" spans="2:12">
@@ -3126,22 +3462,22 @@
         <v>413</v>
       </c>
       <c r="F27" t="s">
-        <v>413</v>
+        <v>429</v>
       </c>
       <c r="G27" t="s">
-        <v>440</v>
+        <v>467</v>
       </c>
       <c r="H27" t="s">
-        <v>441</v>
+        <v>468</v>
       </c>
       <c r="J27" t="s">
-        <v>442</v>
+        <v>470</v>
       </c>
       <c r="K27" t="s">
-        <v>459</v>
+        <v>487</v>
       </c>
       <c r="L27" t="s">
-        <v>459</v>
+        <v>487</v>
       </c>
     </row>
     <row r="28" spans="2:12">
@@ -3155,22 +3491,22 @@
         <v>414</v>
       </c>
       <c r="F28" t="s">
-        <v>414</v>
+        <v>430</v>
       </c>
       <c r="G28" t="s">
-        <v>440</v>
+        <v>467</v>
       </c>
       <c r="H28" t="s">
-        <v>441</v>
+        <v>468</v>
       </c>
       <c r="J28" t="s">
-        <v>442</v>
+        <v>470</v>
       </c>
       <c r="K28" t="s">
-        <v>460</v>
+        <v>488</v>
       </c>
       <c r="L28" t="s">
-        <v>460</v>
+        <v>488</v>
       </c>
     </row>
     <row r="29" spans="2:12">
@@ -3184,22 +3520,22 @@
         <v>415</v>
       </c>
       <c r="F29" t="s">
-        <v>415</v>
+        <v>431</v>
       </c>
       <c r="G29" t="s">
-        <v>440</v>
+        <v>467</v>
       </c>
       <c r="H29" t="s">
-        <v>441</v>
+        <v>468</v>
       </c>
       <c r="J29" t="s">
-        <v>442</v>
+        <v>470</v>
       </c>
       <c r="K29" t="s">
-        <v>461</v>
+        <v>489</v>
       </c>
       <c r="L29" t="s">
-        <v>461</v>
+        <v>489</v>
       </c>
     </row>
     <row r="30" spans="2:12">
@@ -3213,22 +3549,22 @@
         <v>416</v>
       </c>
       <c r="F30" t="s">
-        <v>416</v>
+        <v>432</v>
       </c>
       <c r="G30" t="s">
-        <v>440</v>
+        <v>467</v>
       </c>
       <c r="H30" t="s">
-        <v>441</v>
+        <v>468</v>
       </c>
       <c r="J30" t="s">
-        <v>442</v>
+        <v>470</v>
       </c>
       <c r="K30" t="s">
-        <v>462</v>
+        <v>490</v>
       </c>
       <c r="L30" t="s">
-        <v>462</v>
+        <v>490</v>
       </c>
     </row>
     <row r="31" spans="2:12">
@@ -3242,22 +3578,22 @@
         <v>417</v>
       </c>
       <c r="F31" t="s">
-        <v>417</v>
+        <v>433</v>
       </c>
       <c r="G31" t="s">
-        <v>440</v>
+        <v>467</v>
       </c>
       <c r="H31" t="s">
-        <v>441</v>
+        <v>468</v>
       </c>
       <c r="J31" t="s">
-        <v>442</v>
+        <v>470</v>
       </c>
       <c r="K31" t="s">
-        <v>463</v>
+        <v>491</v>
       </c>
       <c r="L31" t="s">
-        <v>463</v>
+        <v>491</v>
       </c>
     </row>
     <row r="32" spans="2:12">
@@ -3271,22 +3607,22 @@
         <v>418</v>
       </c>
       <c r="F32" t="s">
-        <v>418</v>
+        <v>434</v>
       </c>
       <c r="G32" t="s">
-        <v>440</v>
+        <v>467</v>
       </c>
       <c r="H32" t="s">
-        <v>441</v>
+        <v>468</v>
       </c>
       <c r="J32" t="s">
-        <v>442</v>
+        <v>470</v>
       </c>
       <c r="K32" t="s">
-        <v>464</v>
+        <v>492</v>
       </c>
       <c r="L32" t="s">
-        <v>464</v>
+        <v>492</v>
       </c>
     </row>
     <row r="33" spans="2:12">
@@ -3300,22 +3636,22 @@
         <v>419</v>
       </c>
       <c r="F33" t="s">
-        <v>419</v>
+        <v>435</v>
       </c>
       <c r="G33" t="s">
-        <v>440</v>
+        <v>467</v>
       </c>
       <c r="H33" t="s">
-        <v>441</v>
+        <v>468</v>
       </c>
       <c r="J33" t="s">
-        <v>442</v>
+        <v>470</v>
       </c>
       <c r="K33" t="s">
-        <v>465</v>
+        <v>493</v>
       </c>
       <c r="L33" t="s">
-        <v>465</v>
+        <v>493</v>
       </c>
     </row>
     <row r="34" spans="2:12">
@@ -3329,22 +3665,22 @@
         <v>420</v>
       </c>
       <c r="F34" t="s">
-        <v>420</v>
+        <v>436</v>
       </c>
       <c r="G34" t="s">
-        <v>440</v>
+        <v>467</v>
       </c>
       <c r="H34" t="s">
-        <v>441</v>
+        <v>468</v>
       </c>
       <c r="J34" t="s">
-        <v>442</v>
+        <v>470</v>
       </c>
       <c r="K34" t="s">
-        <v>466</v>
+        <v>494</v>
       </c>
       <c r="L34" t="s">
-        <v>466</v>
+        <v>494</v>
       </c>
     </row>
     <row r="35" spans="2:12">
@@ -3358,22 +3694,22 @@
         <v>421</v>
       </c>
       <c r="F35" t="s">
-        <v>421</v>
+        <v>437</v>
       </c>
       <c r="G35" t="s">
-        <v>440</v>
+        <v>467</v>
       </c>
       <c r="H35" t="s">
-        <v>441</v>
+        <v>468</v>
       </c>
       <c r="J35" t="s">
-        <v>442</v>
+        <v>470</v>
       </c>
       <c r="K35" t="s">
-        <v>467</v>
+        <v>495</v>
       </c>
       <c r="L35" t="s">
-        <v>467</v>
+        <v>495</v>
       </c>
     </row>
     <row r="36" spans="2:12">
@@ -3387,22 +3723,22 @@
         <v>422</v>
       </c>
       <c r="F36" t="s">
-        <v>422</v>
+        <v>438</v>
       </c>
       <c r="G36" t="s">
-        <v>440</v>
+        <v>467</v>
       </c>
       <c r="H36" t="s">
-        <v>441</v>
+        <v>468</v>
       </c>
       <c r="J36" t="s">
-        <v>442</v>
+        <v>470</v>
       </c>
       <c r="K36" t="s">
-        <v>468</v>
+        <v>496</v>
       </c>
       <c r="L36" t="s">
-        <v>468</v>
+        <v>496</v>
       </c>
     </row>
     <row r="37" spans="2:12">
@@ -3416,22 +3752,22 @@
         <v>423</v>
       </c>
       <c r="F37" t="s">
-        <v>423</v>
+        <v>439</v>
       </c>
       <c r="G37" t="s">
-        <v>440</v>
+        <v>467</v>
       </c>
       <c r="H37" t="s">
-        <v>441</v>
+        <v>468</v>
       </c>
       <c r="J37" t="s">
-        <v>442</v>
+        <v>470</v>
       </c>
       <c r="K37" t="s">
-        <v>469</v>
+        <v>497</v>
       </c>
       <c r="L37" t="s">
-        <v>469</v>
+        <v>497</v>
       </c>
     </row>
     <row r="38" spans="2:12">
@@ -3445,22 +3781,22 @@
         <v>424</v>
       </c>
       <c r="F38" t="s">
-        <v>424</v>
+        <v>440</v>
       </c>
       <c r="G38" t="s">
-        <v>440</v>
+        <v>467</v>
       </c>
       <c r="H38" t="s">
-        <v>441</v>
+        <v>468</v>
       </c>
       <c r="J38" t="s">
-        <v>442</v>
+        <v>470</v>
       </c>
       <c r="K38" t="s">
-        <v>470</v>
+        <v>498</v>
       </c>
       <c r="L38" t="s">
-        <v>470</v>
+        <v>498</v>
       </c>
     </row>
     <row r="39" spans="2:12">
@@ -3474,22 +3810,22 @@
         <v>425</v>
       </c>
       <c r="F39" t="s">
-        <v>425</v>
+        <v>441</v>
       </c>
       <c r="G39" t="s">
-        <v>440</v>
+        <v>467</v>
       </c>
       <c r="H39" t="s">
-        <v>441</v>
+        <v>468</v>
       </c>
       <c r="J39" t="s">
-        <v>442</v>
+        <v>470</v>
       </c>
       <c r="K39" t="s">
-        <v>471</v>
+        <v>499</v>
       </c>
       <c r="L39" t="s">
-        <v>471</v>
+        <v>499</v>
       </c>
     </row>
     <row r="40" spans="2:12">
@@ -3503,22 +3839,22 @@
         <v>426</v>
       </c>
       <c r="F40" t="s">
-        <v>426</v>
+        <v>442</v>
       </c>
       <c r="G40" t="s">
-        <v>440</v>
+        <v>467</v>
       </c>
       <c r="H40" t="s">
-        <v>441</v>
+        <v>468</v>
       </c>
       <c r="J40" t="s">
-        <v>442</v>
+        <v>470</v>
       </c>
       <c r="K40" t="s">
-        <v>472</v>
+        <v>500</v>
       </c>
       <c r="L40" t="s">
-        <v>472</v>
+        <v>500</v>
       </c>
     </row>
     <row r="41" spans="2:12">
@@ -3532,22 +3868,22 @@
         <v>427</v>
       </c>
       <c r="F41" t="s">
-        <v>427</v>
+        <v>443</v>
       </c>
       <c r="G41" t="s">
-        <v>440</v>
+        <v>467</v>
       </c>
       <c r="H41" t="s">
-        <v>441</v>
+        <v>468</v>
       </c>
       <c r="J41" t="s">
-        <v>442</v>
+        <v>470</v>
       </c>
       <c r="K41" t="s">
-        <v>473</v>
+        <v>501</v>
       </c>
       <c r="L41" t="s">
-        <v>473</v>
+        <v>501</v>
       </c>
     </row>
     <row r="42" spans="2:12">
@@ -3561,22 +3897,22 @@
         <v>428</v>
       </c>
       <c r="F42" t="s">
-        <v>428</v>
+        <v>444</v>
       </c>
       <c r="G42" t="s">
-        <v>440</v>
+        <v>467</v>
       </c>
       <c r="H42" t="s">
-        <v>441</v>
+        <v>468</v>
       </c>
       <c r="J42" t="s">
-        <v>442</v>
+        <v>470</v>
       </c>
       <c r="K42" t="s">
-        <v>474</v>
+        <v>502</v>
       </c>
       <c r="L42" t="s">
-        <v>474</v>
+        <v>502</v>
       </c>
     </row>
     <row r="43" spans="2:12">
@@ -3590,22 +3926,22 @@
         <v>429</v>
       </c>
       <c r="F43" t="s">
-        <v>429</v>
+        <v>445</v>
       </c>
       <c r="G43" t="s">
-        <v>440</v>
+        <v>467</v>
       </c>
       <c r="H43" t="s">
-        <v>441</v>
+        <v>468</v>
       </c>
       <c r="J43" t="s">
-        <v>442</v>
+        <v>470</v>
       </c>
       <c r="K43" t="s">
-        <v>475</v>
+        <v>503</v>
       </c>
       <c r="L43" t="s">
-        <v>475</v>
+        <v>503</v>
       </c>
     </row>
     <row r="44" spans="2:12">
@@ -3619,22 +3955,22 @@
         <v>430</v>
       </c>
       <c r="F44" t="s">
-        <v>430</v>
+        <v>446</v>
       </c>
       <c r="G44" t="s">
-        <v>440</v>
+        <v>467</v>
       </c>
       <c r="H44" t="s">
-        <v>441</v>
+        <v>468</v>
       </c>
       <c r="J44" t="s">
-        <v>442</v>
+        <v>470</v>
       </c>
       <c r="K44" t="s">
-        <v>476</v>
+        <v>504</v>
       </c>
       <c r="L44" t="s">
-        <v>476</v>
+        <v>504</v>
       </c>
     </row>
     <row r="45" spans="2:12">
@@ -3648,22 +3984,22 @@
         <v>431</v>
       </c>
       <c r="F45" t="s">
-        <v>431</v>
+        <v>447</v>
       </c>
       <c r="G45" t="s">
-        <v>440</v>
+        <v>467</v>
       </c>
       <c r="H45" t="s">
-        <v>441</v>
+        <v>468</v>
       </c>
       <c r="J45" t="s">
-        <v>442</v>
+        <v>470</v>
       </c>
       <c r="K45" t="s">
-        <v>477</v>
+        <v>505</v>
       </c>
       <c r="L45" t="s">
-        <v>477</v>
+        <v>505</v>
       </c>
     </row>
     <row r="46" spans="2:12">
@@ -3677,22 +4013,22 @@
         <v>432</v>
       </c>
       <c r="F46" t="s">
-        <v>432</v>
+        <v>448</v>
       </c>
       <c r="G46" t="s">
-        <v>440</v>
+        <v>467</v>
       </c>
       <c r="H46" t="s">
-        <v>441</v>
+        <v>468</v>
       </c>
       <c r="J46" t="s">
-        <v>442</v>
+        <v>470</v>
       </c>
       <c r="K46" t="s">
-        <v>478</v>
+        <v>506</v>
       </c>
       <c r="L46" t="s">
-        <v>478</v>
+        <v>506</v>
       </c>
     </row>
     <row r="47" spans="2:12">
@@ -3706,22 +4042,22 @@
         <v>433</v>
       </c>
       <c r="F47" t="s">
-        <v>433</v>
+        <v>449</v>
       </c>
       <c r="G47" t="s">
-        <v>440</v>
+        <v>467</v>
       </c>
       <c r="H47" t="s">
-        <v>441</v>
+        <v>468</v>
       </c>
       <c r="J47" t="s">
-        <v>442</v>
+        <v>470</v>
       </c>
       <c r="K47" t="s">
-        <v>479</v>
+        <v>507</v>
       </c>
       <c r="L47" t="s">
-        <v>479</v>
+        <v>507</v>
       </c>
     </row>
     <row r="48" spans="2:12">
@@ -3735,22 +4071,22 @@
         <v>434</v>
       </c>
       <c r="F48" t="s">
-        <v>434</v>
+        <v>450</v>
       </c>
       <c r="G48" t="s">
-        <v>440</v>
+        <v>467</v>
       </c>
       <c r="H48" t="s">
-        <v>441</v>
+        <v>468</v>
       </c>
       <c r="J48" t="s">
-        <v>442</v>
+        <v>470</v>
       </c>
       <c r="K48" t="s">
-        <v>480</v>
+        <v>508</v>
       </c>
       <c r="L48" t="s">
-        <v>480</v>
+        <v>508</v>
       </c>
     </row>
     <row r="49" spans="2:12">
@@ -3764,22 +4100,22 @@
         <v>435</v>
       </c>
       <c r="F49" t="s">
-        <v>435</v>
+        <v>451</v>
       </c>
       <c r="G49" t="s">
-        <v>440</v>
+        <v>467</v>
       </c>
       <c r="H49" t="s">
-        <v>441</v>
+        <v>468</v>
       </c>
       <c r="J49" t="s">
-        <v>442</v>
+        <v>470</v>
       </c>
       <c r="K49" t="s">
-        <v>481</v>
+        <v>509</v>
       </c>
       <c r="L49" t="s">
-        <v>481</v>
+        <v>509</v>
       </c>
     </row>
     <row r="50" spans="2:12">
@@ -3793,22 +4129,22 @@
         <v>436</v>
       </c>
       <c r="F50" t="s">
-        <v>436</v>
+        <v>452</v>
       </c>
       <c r="G50" t="s">
-        <v>440</v>
+        <v>467</v>
       </c>
       <c r="H50" t="s">
-        <v>441</v>
+        <v>468</v>
       </c>
       <c r="J50" t="s">
-        <v>442</v>
+        <v>470</v>
       </c>
       <c r="K50" t="s">
-        <v>482</v>
+        <v>510</v>
       </c>
       <c r="L50" t="s">
-        <v>482</v>
+        <v>510</v>
       </c>
     </row>
     <row r="51" spans="2:12">
@@ -3822,22 +4158,22 @@
         <v>437</v>
       </c>
       <c r="F51" t="s">
-        <v>437</v>
+        <v>453</v>
       </c>
       <c r="G51" t="s">
-        <v>440</v>
+        <v>467</v>
       </c>
       <c r="H51" t="s">
-        <v>441</v>
+        <v>468</v>
       </c>
       <c r="J51" t="s">
-        <v>442</v>
+        <v>470</v>
       </c>
       <c r="K51" t="s">
-        <v>483</v>
+        <v>511</v>
       </c>
       <c r="L51" t="s">
-        <v>483</v>
+        <v>511</v>
       </c>
     </row>
     <row r="52" spans="2:12">
@@ -3851,22 +4187,22 @@
         <v>438</v>
       </c>
       <c r="F52" t="s">
-        <v>438</v>
+        <v>454</v>
       </c>
       <c r="G52" t="s">
-        <v>440</v>
+        <v>467</v>
       </c>
       <c r="H52" t="s">
-        <v>441</v>
+        <v>468</v>
       </c>
       <c r="J52" t="s">
-        <v>442</v>
+        <v>470</v>
       </c>
       <c r="K52" t="s">
-        <v>484</v>
+        <v>512</v>
       </c>
       <c r="L52" t="s">
-        <v>484</v>
+        <v>512</v>
       </c>
     </row>
     <row r="53" spans="2:12">
@@ -3880,22 +4216,970 @@
         <v>439</v>
       </c>
       <c r="F53" t="s">
-        <v>439</v>
+        <v>455</v>
       </c>
       <c r="G53" t="s">
+        <v>467</v>
+      </c>
+      <c r="H53" t="s">
+        <v>468</v>
+      </c>
+      <c r="J53" t="s">
+        <v>470</v>
+      </c>
+      <c r="K53" t="s">
+        <v>513</v>
+      </c>
+      <c r="L53" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="54" spans="2:12">
+      <c r="B54" t="s">
+        <v>396</v>
+      </c>
+      <c r="C54" t="s">
         <v>440</v>
       </c>
-      <c r="H53" t="s">
+      <c r="D54" t="s">
+        <v>440</v>
+      </c>
+      <c r="F54" t="s">
+        <v>456</v>
+      </c>
+      <c r="G54" t="s">
+        <v>467</v>
+      </c>
+      <c r="H54" t="s">
+        <v>469</v>
+      </c>
+      <c r="J54" t="s">
+        <v>470</v>
+      </c>
+      <c r="K54" t="s">
+        <v>514</v>
+      </c>
+      <c r="L54" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="55" spans="2:12">
+      <c r="B55" t="s">
+        <v>396</v>
+      </c>
+      <c r="C55" t="s">
         <v>441</v>
       </c>
-      <c r="J53" t="s">
+      <c r="D55" t="s">
+        <v>441</v>
+      </c>
+      <c r="F55" t="s">
+        <v>457</v>
+      </c>
+      <c r="G55" t="s">
+        <v>467</v>
+      </c>
+      <c r="H55" t="s">
+        <v>469</v>
+      </c>
+      <c r="J55" t="s">
+        <v>470</v>
+      </c>
+      <c r="K55" t="s">
+        <v>515</v>
+      </c>
+      <c r="L55" t="s">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="56" spans="2:12">
+      <c r="B56" t="s">
+        <v>396</v>
+      </c>
+      <c r="C56" t="s">
         <v>442</v>
       </c>
-      <c r="K53" t="s">
-        <v>485</v>
-      </c>
-      <c r="L53" t="s">
-        <v>485</v>
+      <c r="D56" t="s">
+        <v>442</v>
+      </c>
+      <c r="F56" t="s">
+        <v>458</v>
+      </c>
+      <c r="G56" t="s">
+        <v>467</v>
+      </c>
+      <c r="H56" t="s">
+        <v>469</v>
+      </c>
+      <c r="J56" t="s">
+        <v>470</v>
+      </c>
+      <c r="K56" t="s">
+        <v>516</v>
+      </c>
+      <c r="L56" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="57" spans="2:12">
+      <c r="B57" t="s">
+        <v>396</v>
+      </c>
+      <c r="C57" t="s">
+        <v>443</v>
+      </c>
+      <c r="D57" t="s">
+        <v>443</v>
+      </c>
+      <c r="F57" t="s">
+        <v>459</v>
+      </c>
+      <c r="G57" t="s">
+        <v>467</v>
+      </c>
+      <c r="H57" t="s">
+        <v>469</v>
+      </c>
+      <c r="J57" t="s">
+        <v>470</v>
+      </c>
+      <c r="K57" t="s">
+        <v>517</v>
+      </c>
+      <c r="L57" t="s">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="58" spans="2:12">
+      <c r="B58" t="s">
+        <v>396</v>
+      </c>
+      <c r="C58" t="s">
+        <v>444</v>
+      </c>
+      <c r="D58" t="s">
+        <v>444</v>
+      </c>
+      <c r="F58" t="s">
+        <v>460</v>
+      </c>
+      <c r="G58" t="s">
+        <v>467</v>
+      </c>
+      <c r="H58" t="s">
+        <v>469</v>
+      </c>
+      <c r="J58" t="s">
+        <v>470</v>
+      </c>
+      <c r="K58" t="s">
+        <v>518</v>
+      </c>
+      <c r="L58" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="59" spans="2:12">
+      <c r="B59" t="s">
+        <v>396</v>
+      </c>
+      <c r="C59" t="s">
+        <v>445</v>
+      </c>
+      <c r="D59" t="s">
+        <v>445</v>
+      </c>
+      <c r="F59" t="s">
+        <v>461</v>
+      </c>
+      <c r="G59" t="s">
+        <v>467</v>
+      </c>
+      <c r="H59" t="s">
+        <v>469</v>
+      </c>
+      <c r="J59" t="s">
+        <v>470</v>
+      </c>
+      <c r="K59" t="s">
+        <v>519</v>
+      </c>
+      <c r="L59" t="s">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="60" spans="2:12">
+      <c r="B60" t="s">
+        <v>396</v>
+      </c>
+      <c r="C60" t="s">
+        <v>446</v>
+      </c>
+      <c r="D60" t="s">
+        <v>446</v>
+      </c>
+      <c r="F60" t="s">
+        <v>462</v>
+      </c>
+      <c r="G60" t="s">
+        <v>467</v>
+      </c>
+      <c r="H60" t="s">
+        <v>469</v>
+      </c>
+      <c r="J60" t="s">
+        <v>470</v>
+      </c>
+      <c r="K60" t="s">
+        <v>520</v>
+      </c>
+      <c r="L60" t="s">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="61" spans="2:12">
+      <c r="B61" t="s">
+        <v>396</v>
+      </c>
+      <c r="C61" t="s">
+        <v>447</v>
+      </c>
+      <c r="D61" t="s">
+        <v>447</v>
+      </c>
+      <c r="F61" t="s">
+        <v>463</v>
+      </c>
+      <c r="G61" t="s">
+        <v>467</v>
+      </c>
+      <c r="H61" t="s">
+        <v>468</v>
+      </c>
+      <c r="J61" t="s">
+        <v>470</v>
+      </c>
+      <c r="K61" t="s">
+        <v>521</v>
+      </c>
+      <c r="L61" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="62" spans="2:12">
+      <c r="B62" t="s">
+        <v>396</v>
+      </c>
+      <c r="C62" t="s">
+        <v>448</v>
+      </c>
+      <c r="D62" t="s">
+        <v>448</v>
+      </c>
+      <c r="F62" t="s">
+        <v>464</v>
+      </c>
+      <c r="G62" t="s">
+        <v>467</v>
+      </c>
+      <c r="H62" t="s">
+        <v>469</v>
+      </c>
+      <c r="J62" t="s">
+        <v>470</v>
+      </c>
+      <c r="K62" t="s">
+        <v>522</v>
+      </c>
+      <c r="L62" t="s">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="63" spans="2:12">
+      <c r="B63" t="s">
+        <v>396</v>
+      </c>
+      <c r="C63" t="s">
+        <v>449</v>
+      </c>
+      <c r="D63" t="s">
+        <v>449</v>
+      </c>
+      <c r="F63" t="s">
+        <v>465</v>
+      </c>
+      <c r="G63" t="s">
+        <v>467</v>
+      </c>
+      <c r="H63" t="s">
+        <v>469</v>
+      </c>
+      <c r="J63" t="s">
+        <v>470</v>
+      </c>
+      <c r="K63" t="s">
+        <v>523</v>
+      </c>
+      <c r="L63" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="64" spans="2:12">
+      <c r="B64" t="s">
+        <v>396</v>
+      </c>
+      <c r="C64" t="s">
+        <v>450</v>
+      </c>
+      <c r="D64" t="s">
+        <v>450</v>
+      </c>
+      <c r="F64" t="s">
+        <v>466</v>
+      </c>
+      <c r="G64" t="s">
+        <v>467</v>
+      </c>
+      <c r="H64" t="s">
+        <v>469</v>
+      </c>
+      <c r="J64" t="s">
+        <v>470</v>
+      </c>
+      <c r="K64" t="s">
+        <v>524</v>
+      </c>
+      <c r="L64" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="65" spans="2:12">
+      <c r="B65" t="s">
+        <v>396</v>
+      </c>
+      <c r="C65" t="s">
+        <v>451</v>
+      </c>
+      <c r="D65" t="s">
+        <v>451</v>
+      </c>
+      <c r="F65" t="s">
+        <v>412</v>
+      </c>
+      <c r="G65" t="s">
+        <v>467</v>
+      </c>
+      <c r="H65" t="s">
+        <v>468</v>
+      </c>
+      <c r="J65" t="s">
+        <v>470</v>
+      </c>
+      <c r="K65" t="s">
+        <v>525</v>
+      </c>
+      <c r="L65" t="s">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="66" spans="2:12">
+      <c r="B66" t="s">
+        <v>396</v>
+      </c>
+      <c r="C66" t="s">
+        <v>452</v>
+      </c>
+      <c r="D66" t="s">
+        <v>452</v>
+      </c>
+      <c r="F66" t="s">
+        <v>413</v>
+      </c>
+      <c r="G66" t="s">
+        <v>467</v>
+      </c>
+      <c r="H66" t="s">
+        <v>468</v>
+      </c>
+      <c r="J66" t="s">
+        <v>470</v>
+      </c>
+      <c r="K66" t="s">
+        <v>526</v>
+      </c>
+      <c r="L66" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="67" spans="2:12">
+      <c r="B67" t="s">
+        <v>396</v>
+      </c>
+      <c r="C67" t="s">
+        <v>453</v>
+      </c>
+      <c r="D67" t="s">
+        <v>453</v>
+      </c>
+      <c r="F67" t="s">
+        <v>414</v>
+      </c>
+      <c r="G67" t="s">
+        <v>467</v>
+      </c>
+      <c r="H67" t="s">
+        <v>468</v>
+      </c>
+      <c r="J67" t="s">
+        <v>470</v>
+      </c>
+      <c r="K67" t="s">
+        <v>527</v>
+      </c>
+      <c r="L67" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="68" spans="2:12">
+      <c r="B68" t="s">
+        <v>396</v>
+      </c>
+      <c r="C68" t="s">
+        <v>454</v>
+      </c>
+      <c r="D68" t="s">
+        <v>454</v>
+      </c>
+      <c r="F68" t="s">
+        <v>415</v>
+      </c>
+      <c r="G68" t="s">
+        <v>467</v>
+      </c>
+      <c r="H68" t="s">
+        <v>468</v>
+      </c>
+      <c r="J68" t="s">
+        <v>470</v>
+      </c>
+      <c r="K68" t="s">
+        <v>528</v>
+      </c>
+      <c r="L68" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="69" spans="2:12">
+      <c r="B69" t="s">
+        <v>396</v>
+      </c>
+      <c r="C69" t="s">
+        <v>455</v>
+      </c>
+      <c r="D69" t="s">
+        <v>455</v>
+      </c>
+      <c r="F69" t="s">
+        <v>416</v>
+      </c>
+      <c r="G69" t="s">
+        <v>467</v>
+      </c>
+      <c r="H69" t="s">
+        <v>468</v>
+      </c>
+      <c r="J69" t="s">
+        <v>470</v>
+      </c>
+      <c r="K69" t="s">
+        <v>529</v>
+      </c>
+      <c r="L69" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="70" spans="2:12">
+      <c r="B70" t="s">
+        <v>396</v>
+      </c>
+      <c r="C70" t="s">
+        <v>456</v>
+      </c>
+      <c r="D70" t="s">
+        <v>456</v>
+      </c>
+      <c r="F70" t="s">
+        <v>417</v>
+      </c>
+      <c r="G70" t="s">
+        <v>467</v>
+      </c>
+      <c r="H70" t="s">
+        <v>469</v>
+      </c>
+      <c r="J70" t="s">
+        <v>470</v>
+      </c>
+      <c r="K70" t="s">
+        <v>530</v>
+      </c>
+      <c r="L70" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="71" spans="2:12">
+      <c r="B71" t="s">
+        <v>396</v>
+      </c>
+      <c r="C71" t="s">
+        <v>457</v>
+      </c>
+      <c r="D71" t="s">
+        <v>457</v>
+      </c>
+      <c r="F71" t="s">
+        <v>418</v>
+      </c>
+      <c r="G71" t="s">
+        <v>467</v>
+      </c>
+      <c r="H71" t="s">
+        <v>468</v>
+      </c>
+      <c r="J71" t="s">
+        <v>470</v>
+      </c>
+      <c r="K71" t="s">
+        <v>531</v>
+      </c>
+      <c r="L71" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="72" spans="2:12">
+      <c r="B72" t="s">
+        <v>396</v>
+      </c>
+      <c r="C72" t="s">
+        <v>458</v>
+      </c>
+      <c r="D72" t="s">
+        <v>458</v>
+      </c>
+      <c r="F72" t="s">
+        <v>419</v>
+      </c>
+      <c r="G72" t="s">
+        <v>467</v>
+      </c>
+      <c r="H72" t="s">
+        <v>468</v>
+      </c>
+      <c r="J72" t="s">
+        <v>470</v>
+      </c>
+      <c r="K72" t="s">
+        <v>532</v>
+      </c>
+      <c r="L72" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="73" spans="2:12">
+      <c r="B73" t="s">
+        <v>396</v>
+      </c>
+      <c r="C73" t="s">
+        <v>459</v>
+      </c>
+      <c r="D73" t="s">
+        <v>459</v>
+      </c>
+      <c r="F73" t="s">
+        <v>420</v>
+      </c>
+      <c r="G73" t="s">
+        <v>467</v>
+      </c>
+      <c r="H73" t="s">
+        <v>468</v>
+      </c>
+      <c r="J73" t="s">
+        <v>470</v>
+      </c>
+      <c r="K73" t="s">
+        <v>533</v>
+      </c>
+      <c r="L73" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="74" spans="2:12">
+      <c r="B74" t="s">
+        <v>396</v>
+      </c>
+      <c r="C74" t="s">
+        <v>460</v>
+      </c>
+      <c r="D74" t="s">
+        <v>460</v>
+      </c>
+      <c r="F74" t="s">
+        <v>421</v>
+      </c>
+      <c r="G74" t="s">
+        <v>467</v>
+      </c>
+      <c r="H74" t="s">
+        <v>468</v>
+      </c>
+      <c r="J74" t="s">
+        <v>470</v>
+      </c>
+      <c r="K74" t="s">
+        <v>534</v>
+      </c>
+      <c r="L74" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="75" spans="2:12">
+      <c r="B75" t="s">
+        <v>396</v>
+      </c>
+      <c r="C75" t="s">
+        <v>461</v>
+      </c>
+      <c r="D75" t="s">
+        <v>461</v>
+      </c>
+      <c r="F75" t="s">
+        <v>422</v>
+      </c>
+      <c r="G75" t="s">
+        <v>467</v>
+      </c>
+      <c r="H75" t="s">
+        <v>469</v>
+      </c>
+      <c r="J75" t="s">
+        <v>470</v>
+      </c>
+      <c r="K75" t="s">
+        <v>535</v>
+      </c>
+      <c r="L75" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="76" spans="2:12">
+      <c r="B76" t="s">
+        <v>396</v>
+      </c>
+      <c r="C76" t="s">
+        <v>462</v>
+      </c>
+      <c r="D76" t="s">
+        <v>462</v>
+      </c>
+      <c r="F76" t="s">
+        <v>423</v>
+      </c>
+      <c r="G76" t="s">
+        <v>467</v>
+      </c>
+      <c r="H76" t="s">
+        <v>469</v>
+      </c>
+      <c r="J76" t="s">
+        <v>470</v>
+      </c>
+      <c r="K76" t="s">
+        <v>536</v>
+      </c>
+      <c r="L76" t="s">
+        <v>536</v>
+      </c>
+    </row>
+    <row r="77" spans="2:12">
+      <c r="B77" t="s">
+        <v>396</v>
+      </c>
+      <c r="C77" t="s">
+        <v>463</v>
+      </c>
+      <c r="D77" t="s">
+        <v>463</v>
+      </c>
+      <c r="F77" t="s">
+        <v>424</v>
+      </c>
+      <c r="G77" t="s">
+        <v>467</v>
+      </c>
+      <c r="H77" t="s">
+        <v>469</v>
+      </c>
+      <c r="J77" t="s">
+        <v>470</v>
+      </c>
+      <c r="K77" t="s">
+        <v>537</v>
+      </c>
+      <c r="L77" t="s">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="78" spans="2:12">
+      <c r="B78" t="s">
+        <v>396</v>
+      </c>
+      <c r="C78" t="s">
+        <v>464</v>
+      </c>
+      <c r="D78" t="s">
+        <v>464</v>
+      </c>
+      <c r="F78" t="s">
+        <v>425</v>
+      </c>
+      <c r="G78" t="s">
+        <v>467</v>
+      </c>
+      <c r="H78" t="s">
+        <v>469</v>
+      </c>
+      <c r="J78" t="s">
+        <v>470</v>
+      </c>
+      <c r="K78" t="s">
+        <v>538</v>
+      </c>
+      <c r="L78" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="79" spans="2:12">
+      <c r="B79" t="s">
+        <v>396</v>
+      </c>
+      <c r="C79" t="s">
+        <v>465</v>
+      </c>
+      <c r="D79" t="s">
+        <v>465</v>
+      </c>
+      <c r="F79" t="s">
+        <v>426</v>
+      </c>
+      <c r="G79" t="s">
+        <v>467</v>
+      </c>
+      <c r="H79" t="s">
+        <v>469</v>
+      </c>
+      <c r="J79" t="s">
+        <v>470</v>
+      </c>
+      <c r="K79" t="s">
+        <v>539</v>
+      </c>
+      <c r="L79" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="80" spans="2:12">
+      <c r="B80" t="s">
+        <v>396</v>
+      </c>
+      <c r="C80" t="s">
+        <v>466</v>
+      </c>
+      <c r="D80" t="s">
+        <v>466</v>
+      </c>
+      <c r="F80" t="s">
+        <v>427</v>
+      </c>
+      <c r="G80" t="s">
+        <v>467</v>
+      </c>
+      <c r="H80" t="s">
+        <v>469</v>
+      </c>
+      <c r="J80" t="s">
+        <v>470</v>
+      </c>
+      <c r="K80" t="s">
+        <v>540</v>
+      </c>
+      <c r="L80" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="81" spans="10:12">
+      <c r="J81" t="s">
+        <v>470</v>
+      </c>
+      <c r="K81" t="s">
+        <v>541</v>
+      </c>
+      <c r="L81" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="82" spans="10:12">
+      <c r="J82" t="s">
+        <v>470</v>
+      </c>
+      <c r="K82" t="s">
+        <v>542</v>
+      </c>
+      <c r="L82" t="s">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="83" spans="10:12">
+      <c r="J83" t="s">
+        <v>470</v>
+      </c>
+      <c r="K83" t="s">
+        <v>543</v>
+      </c>
+      <c r="L83" t="s">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="84" spans="10:12">
+      <c r="J84" t="s">
+        <v>470</v>
+      </c>
+      <c r="K84" t="s">
+        <v>544</v>
+      </c>
+      <c r="L84" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="85" spans="10:12">
+      <c r="J85" t="s">
+        <v>470</v>
+      </c>
+      <c r="K85" t="s">
+        <v>545</v>
+      </c>
+      <c r="L85" t="s">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="86" spans="10:12">
+      <c r="J86" t="s">
+        <v>470</v>
+      </c>
+      <c r="K86" t="s">
+        <v>546</v>
+      </c>
+      <c r="L86" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="87" spans="10:12">
+      <c r="J87" t="s">
+        <v>470</v>
+      </c>
+      <c r="K87" t="s">
+        <v>547</v>
+      </c>
+      <c r="L87" t="s">
+        <v>547</v>
+      </c>
+    </row>
+    <row r="88" spans="10:12">
+      <c r="J88" t="s">
+        <v>470</v>
+      </c>
+      <c r="K88" t="s">
+        <v>548</v>
+      </c>
+      <c r="L88" t="s">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="89" spans="10:12">
+      <c r="J89" t="s">
+        <v>470</v>
+      </c>
+      <c r="K89" t="s">
+        <v>549</v>
+      </c>
+      <c r="L89" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="90" spans="10:12">
+      <c r="J90" t="s">
+        <v>470</v>
+      </c>
+      <c r="K90" t="s">
+        <v>550</v>
+      </c>
+      <c r="L90" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="91" spans="10:12">
+      <c r="J91" t="s">
+        <v>470</v>
+      </c>
+      <c r="K91" t="s">
+        <v>551</v>
+      </c>
+      <c r="L91" t="s">
+        <v>551</v>
+      </c>
+    </row>
+    <row r="92" spans="10:12">
+      <c r="J92" t="s">
+        <v>470</v>
+      </c>
+      <c r="K92" t="s">
+        <v>552</v>
+      </c>
+      <c r="L92" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="93" spans="10:12">
+      <c r="J93" t="s">
+        <v>470</v>
+      </c>
+      <c r="K93" t="s">
+        <v>553</v>
+      </c>
+      <c r="L93" t="s">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="94" spans="10:12">
+      <c r="J94" t="s">
+        <v>470</v>
+      </c>
+      <c r="K94" t="s">
+        <v>554</v>
+      </c>
+      <c r="L94" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="95" spans="10:12">
+      <c r="J95" t="s">
+        <v>470</v>
+      </c>
+      <c r="K95" t="s">
+        <v>555</v>
+      </c>
+      <c r="L95" t="s">
+        <v>555</v>
       </c>
     </row>
   </sheetData>
@@ -25748,16 +27032,16 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14D1024C-CB50-4338-8309-6783BE3B28B4}">
-  <dimension ref="B9:H53"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D236420-6A83-4679-9382-901650BE12E7}">
+  <dimension ref="B9:H95"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
     <row r="9" spans="2:8">
       <c r="B9" t="s">
-        <v>486</v>
+        <v>556</v>
       </c>
       <c r="F9" t="s">
-        <v>486</v>
+        <v>556</v>
       </c>
     </row>
     <row r="10" spans="2:8">
@@ -25765,19 +27049,19 @@
         <v>389</v>
       </c>
       <c r="C10" t="s">
-        <v>487</v>
+        <v>557</v>
       </c>
       <c r="D10" t="s">
-        <v>488</v>
+        <v>558</v>
       </c>
       <c r="F10" t="s">
         <v>389</v>
       </c>
       <c r="G10" t="s">
-        <v>487</v>
+        <v>557</v>
       </c>
       <c r="H10" t="s">
-        <v>488</v>
+        <v>558</v>
       </c>
     </row>
     <row r="11" spans="2:8">
@@ -25791,7 +27075,7 @@
         <v>18.420983798347297</v>
       </c>
       <c r="F11" t="s">
-        <v>489</v>
+        <v>559</v>
       </c>
       <c r="G11">
         <v>45.288705409625472</v>
@@ -25811,7 +27095,7 @@
         <v>15.903205816155046</v>
       </c>
       <c r="F12" t="s">
-        <v>490</v>
+        <v>560</v>
       </c>
       <c r="G12">
         <v>43.756388757532321</v>
@@ -25831,7 +27115,7 @@
         <v>15.754697507990151</v>
       </c>
       <c r="F13" t="s">
-        <v>491</v>
+        <v>561</v>
       </c>
       <c r="G13">
         <v>44.207396025652962</v>
@@ -25851,7 +27135,7 @@
         <v>16.41378481811703</v>
       </c>
       <c r="F14" t="s">
-        <v>492</v>
+        <v>562</v>
       </c>
       <c r="G14">
         <v>45.452492401724257</v>
@@ -25871,7 +27155,7 @@
         <v>14.166639022574504</v>
       </c>
       <c r="F15" t="s">
-        <v>493</v>
+        <v>563</v>
       </c>
       <c r="G15">
         <v>45.137590945224346</v>
@@ -25891,7 +27175,7 @@
         <v>15.105276725972995</v>
       </c>
       <c r="F16" t="s">
-        <v>494</v>
+        <v>564</v>
       </c>
       <c r="G16">
         <v>44.993014847588817</v>
@@ -25911,7 +27195,7 @@
         <v>16.500996377679218</v>
       </c>
       <c r="F17" t="s">
-        <v>495</v>
+        <v>565</v>
       </c>
       <c r="G17">
         <v>43.600259258254958</v>
@@ -25931,7 +27215,7 @@
         <v>16.501279071484671</v>
       </c>
       <c r="F18" t="s">
-        <v>496</v>
+        <v>566</v>
       </c>
       <c r="G18">
         <v>43.60043328704915</v>
@@ -25951,7 +27235,7 @@
         <v>14.563904567364178</v>
       </c>
       <c r="F19" t="s">
-        <v>497</v>
+        <v>567</v>
       </c>
       <c r="G19">
         <v>45.316184595349739</v>
@@ -25971,7 +27255,7 @@
         <v>14.564190054501609</v>
       </c>
       <c r="F20" t="s">
-        <v>498</v>
+        <v>568</v>
       </c>
       <c r="G20">
         <v>45.31636366839107</v>
@@ -25991,7 +27275,7 @@
         <v>15.869401606746242</v>
       </c>
       <c r="F21" t="s">
-        <v>499</v>
+        <v>569</v>
       </c>
       <c r="G21">
         <v>45.681428265735541</v>
@@ -26011,7 +27295,7 @@
         <v>16.111889141850742</v>
       </c>
       <c r="F22" t="s">
-        <v>500</v>
+        <v>570</v>
       </c>
       <c r="G22">
         <v>45.667427381860662</v>
@@ -26031,7 +27315,7 @@
         <v>16.162877551551272</v>
       </c>
       <c r="F23" t="s">
-        <v>501</v>
+        <v>571</v>
       </c>
       <c r="G23">
         <v>45.876171942571233</v>
@@ -26051,7 +27335,7 @@
         <v>18.663329039744493</v>
       </c>
       <c r="F24" t="s">
-        <v>502</v>
+        <v>572</v>
       </c>
       <c r="G24">
         <v>45.473186839980002</v>
@@ -26071,7 +27355,7 @@
         <v>16.913620388699012</v>
       </c>
       <c r="F25" t="s">
-        <v>503</v>
+        <v>573</v>
       </c>
       <c r="G25">
         <v>45.448081289056574</v>
@@ -26082,7 +27366,7 @@
     </row>
     <row r="26" spans="2:8">
       <c r="B26" t="s">
-        <v>412</v>
+        <v>428</v>
       </c>
       <c r="C26">
         <v>43.48127785283075</v>
@@ -26091,7 +27375,7 @@
         <v>16.710820911101308</v>
       </c>
       <c r="F26" t="s">
-        <v>504</v>
+        <v>574</v>
       </c>
       <c r="G26">
         <v>43.48127785283075</v>
@@ -26102,7 +27386,7 @@
     </row>
     <row r="27" spans="2:8">
       <c r="B27" t="s">
-        <v>413</v>
+        <v>429</v>
       </c>
       <c r="C27">
         <v>43.972461105244413</v>
@@ -26111,7 +27395,7 @@
         <v>15.9785336822579</v>
       </c>
       <c r="F27" t="s">
-        <v>505</v>
+        <v>575</v>
       </c>
       <c r="G27">
         <v>43.972461105244413</v>
@@ -26122,7 +27406,7 @@
     </row>
     <row r="28" spans="2:8">
       <c r="B28" t="s">
-        <v>414</v>
+        <v>430</v>
       </c>
       <c r="C28">
         <v>45.181638277791002</v>
@@ -26131,7 +27415,7 @@
         <v>13.84520419692222</v>
       </c>
       <c r="F28" t="s">
-        <v>506</v>
+        <v>576</v>
       </c>
       <c r="G28">
         <v>45.181638277791002</v>
@@ -26142,7 +27426,7 @@
     </row>
     <row r="29" spans="2:8">
       <c r="B29" t="s">
-        <v>415</v>
+        <v>431</v>
       </c>
       <c r="C29">
         <v>45.439563689112191</v>
@@ -26151,7 +27435,7 @@
         <v>14.346597512358873</v>
       </c>
       <c r="F29" t="s">
-        <v>507</v>
+        <v>577</v>
       </c>
       <c r="G29">
         <v>45.439563689112191</v>
@@ -26162,7 +27446,7 @@
     </row>
     <row r="30" spans="2:8">
       <c r="B30" t="s">
-        <v>416</v>
+        <v>432</v>
       </c>
       <c r="C30">
         <v>45.205827771951057</v>
@@ -26171,7 +27455,7 @@
         <v>15.106238717929074</v>
       </c>
       <c r="F30" t="s">
-        <v>508</v>
+        <v>578</v>
       </c>
       <c r="G30">
         <v>45.205827771951057</v>
@@ -26182,7 +27466,7 @@
     </row>
     <row r="31" spans="2:8">
       <c r="B31" t="s">
-        <v>417</v>
+        <v>433</v>
       </c>
       <c r="C31">
         <v>44.548836666301071</v>
@@ -26191,7 +27475,7 @@
         <v>15.345859676082814</v>
       </c>
       <c r="F31" t="s">
-        <v>509</v>
+        <v>579</v>
       </c>
       <c r="G31">
         <v>44.548836666301071</v>
@@ -26202,7 +27486,7 @@
     </row>
     <row r="32" spans="2:8">
       <c r="B32" t="s">
-        <v>418</v>
+        <v>434</v>
       </c>
       <c r="C32">
         <v>44.811542804850241</v>
@@ -26211,7 +27495,7 @@
         <v>15.644380101618548</v>
       </c>
       <c r="F32" t="s">
-        <v>510</v>
+        <v>580</v>
       </c>
       <c r="G32">
         <v>44.811542804850241</v>
@@ -26222,7 +27506,7 @@
     </row>
     <row r="33" spans="2:8">
       <c r="B33" t="s">
-        <v>419</v>
+        <v>435</v>
       </c>
       <c r="C33">
         <v>45.397334647918726</v>
@@ -26231,7 +27515,7 @@
         <v>15.93302507721782</v>
       </c>
       <c r="F33" t="s">
-        <v>511</v>
+        <v>581</v>
       </c>
       <c r="G33">
         <v>45.397334647918726</v>
@@ -26242,7 +27526,7 @@
     </row>
     <row r="34" spans="2:8">
       <c r="B34" t="s">
-        <v>420</v>
+        <v>436</v>
       </c>
       <c r="C34">
         <v>46.371362638644037</v>
@@ -26251,7 +27535,7 @@
         <v>16.406716802789003</v>
       </c>
       <c r="F34" t="s">
-        <v>512</v>
+        <v>582</v>
       </c>
       <c r="G34">
         <v>46.371362638644037</v>
@@ -26262,7 +27546,7 @@
     </row>
     <row r="35" spans="2:8">
       <c r="B35" t="s">
-        <v>421</v>
+        <v>437</v>
       </c>
       <c r="C35">
         <v>45.965407015802704</v>
@@ -26271,7 +27555,7 @@
         <v>16.275783798608799</v>
       </c>
       <c r="F35" t="s">
-        <v>513</v>
+        <v>583</v>
       </c>
       <c r="G35">
         <v>45.965407015802704</v>
@@ -26282,7 +27566,7 @@
     </row>
     <row r="36" spans="2:8">
       <c r="B36" t="s">
-        <v>422</v>
+        <v>438</v>
       </c>
       <c r="C36">
         <v>45.062394360999221</v>
@@ -26291,7 +27575,7 @@
         <v>18.886896369105667</v>
       </c>
       <c r="F36" t="s">
-        <v>514</v>
+        <v>584</v>
       </c>
       <c r="G36">
         <v>45.062394360999221</v>
@@ -26302,7 +27586,7 @@
     </row>
     <row r="37" spans="2:8">
       <c r="B37" t="s">
-        <v>423</v>
+        <v>439</v>
       </c>
       <c r="C37">
         <v>45.625896984677652</v>
@@ -26311,7 +27595,7 @@
         <v>18.700291150137662</v>
       </c>
       <c r="F37" t="s">
-        <v>515</v>
+        <v>585</v>
       </c>
       <c r="G37">
         <v>45.625896984677652</v>
@@ -26322,7 +27606,7 @@
     </row>
     <row r="38" spans="2:8">
       <c r="B38" t="s">
-        <v>424</v>
+        <v>440</v>
       </c>
       <c r="C38">
         <v>45.414393829297886</v>
@@ -26331,7 +27615,7 @@
         <v>17.711632151803759</v>
       </c>
       <c r="F38" t="s">
-        <v>516</v>
+        <v>586</v>
       </c>
       <c r="G38">
         <v>45.414393829297886</v>
@@ -26342,7 +27626,7 @@
     </row>
     <row r="39" spans="2:8">
       <c r="B39" t="s">
-        <v>425</v>
+        <v>441</v>
       </c>
       <c r="C39">
         <v>45.909013725374528</v>
@@ -26351,7 +27635,7 @@
         <v>17.200308658553954</v>
       </c>
       <c r="F39" t="s">
-        <v>517</v>
+        <v>587</v>
       </c>
       <c r="G39">
         <v>45.909013725374528</v>
@@ -26362,7 +27646,7 @@
     </row>
     <row r="40" spans="2:8">
       <c r="B40" t="s">
-        <v>426</v>
+        <v>442</v>
       </c>
       <c r="C40">
         <v>45.54209383479413</v>
@@ -26371,7 +27655,7 @@
         <v>16.669818039986271</v>
       </c>
       <c r="F40" t="s">
-        <v>518</v>
+        <v>588</v>
       </c>
       <c r="G40">
         <v>45.54209383479413</v>
@@ -26382,7 +27666,7 @@
     </row>
     <row r="41" spans="2:8">
       <c r="B41" t="s">
-        <v>427</v>
+        <v>443</v>
       </c>
       <c r="C41">
         <v>42.947075227327844</v>
@@ -26391,7 +27675,7 @@
         <v>17.600065674778687</v>
       </c>
       <c r="F41" t="s">
-        <v>519</v>
+        <v>589</v>
       </c>
       <c r="G41">
         <v>42.947075227327844</v>
@@ -26402,7 +27686,7 @@
     </row>
     <row r="42" spans="2:8">
       <c r="B42" t="s">
-        <v>428</v>
+        <v>444</v>
       </c>
       <c r="C42">
         <v>43.618932251323209</v>
@@ -26411,7 +27695,7 @@
         <v>16.579162967152065</v>
       </c>
       <c r="F42" t="s">
-        <v>520</v>
+        <v>590</v>
       </c>
       <c r="G42">
         <v>43.618932251323209</v>
@@ -26422,7 +27706,7 @@
     </row>
     <row r="43" spans="2:8">
       <c r="B43" t="s">
-        <v>429</v>
+        <v>445</v>
       </c>
       <c r="C43">
         <v>45.07863711613124</v>
@@ -26431,7 +27715,7 @@
         <v>13.906762304385827</v>
       </c>
       <c r="F43" t="s">
-        <v>521</v>
+        <v>591</v>
       </c>
       <c r="G43">
         <v>45.07863711613124</v>
@@ -26442,7 +27726,7 @@
     </row>
     <row r="44" spans="2:8">
       <c r="B44" t="s">
-        <v>430</v>
+        <v>446</v>
       </c>
       <c r="C44">
         <v>45.331946195599471</v>
@@ -26451,7 +27735,7 @@
         <v>14.483886991838087</v>
       </c>
       <c r="F44" t="s">
-        <v>522</v>
+        <v>592</v>
       </c>
       <c r="G44">
         <v>45.331946195599471</v>
@@ -26462,7 +27746,7 @@
     </row>
     <row r="45" spans="2:8">
       <c r="B45" t="s">
-        <v>431</v>
+        <v>447</v>
       </c>
       <c r="C45">
         <v>44.012498899877137</v>
@@ -26471,7 +27755,7 @@
         <v>15.809377084060609</v>
       </c>
       <c r="F45" t="s">
-        <v>523</v>
+        <v>593</v>
       </c>
       <c r="G45">
         <v>44.012498899877137</v>
@@ -26482,7 +27766,7 @@
     </row>
     <row r="46" spans="2:8">
       <c r="B46" t="s">
-        <v>432</v>
+        <v>448</v>
       </c>
       <c r="C46">
         <v>44.523125556136428</v>
@@ -26491,7 +27775,7 @@
         <v>15.164471200835765</v>
       </c>
       <c r="F46" t="s">
-        <v>524</v>
+        <v>594</v>
       </c>
       <c r="G46">
         <v>44.523125556136428</v>
@@ -26502,7 +27786,7 @@
     </row>
     <row r="47" spans="2:8">
       <c r="B47" t="s">
-        <v>433</v>
+        <v>449</v>
       </c>
       <c r="C47">
         <v>44.348016883150542</v>
@@ -26511,7 +27795,7 @@
         <v>15.782157995565388</v>
       </c>
       <c r="F47" t="s">
-        <v>525</v>
+        <v>595</v>
       </c>
       <c r="G47">
         <v>44.348016883150542</v>
@@ -26522,7 +27806,7 @@
     </row>
     <row r="48" spans="2:8">
       <c r="B48" t="s">
-        <v>434</v>
+        <v>450</v>
       </c>
       <c r="C48">
         <v>45.357187206013201</v>
@@ -26531,7 +27815,7 @@
         <v>18.335316155297647</v>
       </c>
       <c r="F48" t="s">
-        <v>526</v>
+        <v>596</v>
       </c>
       <c r="G48">
         <v>45.357187206013201</v>
@@ -26542,7 +27826,7 @@
     </row>
     <row r="49" spans="2:8">
       <c r="B49" t="s">
-        <v>435</v>
+        <v>451</v>
       </c>
       <c r="C49">
         <v>45.493689175149086</v>
@@ -26551,7 +27835,7 @@
         <v>18.766510818285862</v>
       </c>
       <c r="F49" t="s">
-        <v>527</v>
+        <v>597</v>
       </c>
       <c r="G49">
         <v>45.493689175149086</v>
@@ -26562,7 +27846,7 @@
     </row>
     <row r="50" spans="2:8">
       <c r="B50" t="s">
-        <v>436</v>
+        <v>452</v>
       </c>
       <c r="C50">
         <v>45.640389174848501</v>
@@ -26571,7 +27855,7 @@
         <v>16.644419020683017</v>
       </c>
       <c r="F50" t="s">
-        <v>528</v>
+        <v>598</v>
       </c>
       <c r="G50">
         <v>45.640389174848501</v>
@@ -26582,7 +27866,7 @@
     </row>
     <row r="51" spans="2:8">
       <c r="B51" t="s">
-        <v>437</v>
+        <v>453</v>
       </c>
       <c r="C51">
         <v>46.005205111639626</v>
@@ -26591,7 +27875,7 @@
         <v>16.058351137930462</v>
       </c>
       <c r="F51" t="s">
-        <v>529</v>
+        <v>599</v>
       </c>
       <c r="G51">
         <v>46.005205111639626</v>
@@ -26602,7 +27886,7 @@
     </row>
     <row r="52" spans="2:8">
       <c r="B52" t="s">
-        <v>438</v>
+        <v>454</v>
       </c>
       <c r="C52">
         <v>46.374206998637192</v>
@@ -26611,7 +27895,7 @@
         <v>16.448711926621812</v>
       </c>
       <c r="F52" t="s">
-        <v>530</v>
+        <v>600</v>
       </c>
       <c r="G52">
         <v>46.374206998637192</v>
@@ -26622,7 +27906,7 @@
     </row>
     <row r="53" spans="2:8">
       <c r="B53" t="s">
-        <v>439</v>
+        <v>455</v>
       </c>
       <c r="C53">
         <v>45.926508069000413</v>
@@ -26631,13 +27915,718 @@
         <v>16.916722421469085</v>
       </c>
       <c r="F53" t="s">
-        <v>531</v>
+        <v>601</v>
       </c>
       <c r="G53">
         <v>45.926508069000413</v>
       </c>
       <c r="H53">
         <v>16.916722421469085</v>
+      </c>
+    </row>
+    <row r="54" spans="2:8">
+      <c r="B54" t="s">
+        <v>456</v>
+      </c>
+      <c r="C54">
+        <v>44.454932217252427</v>
+      </c>
+      <c r="D54">
+        <v>13.803928694655268</v>
+      </c>
+      <c r="F54" t="s">
+        <v>602</v>
+      </c>
+      <c r="G54">
+        <v>44.454932217252427</v>
+      </c>
+      <c r="H54">
+        <v>13.803928694655268</v>
+      </c>
+    </row>
+    <row r="55" spans="2:8">
+      <c r="B55" t="s">
+        <v>457</v>
+      </c>
+      <c r="C55">
+        <v>42.466360025001833</v>
+      </c>
+      <c r="D55">
+        <v>16.828384390409024</v>
+      </c>
+      <c r="F55" t="s">
+        <v>603</v>
+      </c>
+      <c r="G55">
+        <v>42.466360025001833</v>
+      </c>
+      <c r="H55">
+        <v>16.828384390409024</v>
+      </c>
+    </row>
+    <row r="56" spans="2:8">
+      <c r="B56" t="s">
+        <v>458</v>
+      </c>
+      <c r="C56">
+        <v>42.125213525162977</v>
+      </c>
+      <c r="D56">
+        <v>18.270796243376044</v>
+      </c>
+      <c r="F56" t="s">
+        <v>604</v>
+      </c>
+      <c r="G56">
+        <v>42.125213525162977</v>
+      </c>
+      <c r="H56">
+        <v>18.270796243376044</v>
+      </c>
+    </row>
+    <row r="57" spans="2:8">
+      <c r="B57" t="s">
+        <v>459</v>
+      </c>
+      <c r="C57">
+        <v>42.538207099784479</v>
+      </c>
+      <c r="D57">
+        <v>17.506483224613337</v>
+      </c>
+      <c r="F57" t="s">
+        <v>605</v>
+      </c>
+      <c r="G57">
+        <v>42.538207099784479</v>
+      </c>
+      <c r="H57">
+        <v>17.506483224613337</v>
+      </c>
+    </row>
+    <row r="58" spans="2:8">
+      <c r="B58" t="s">
+        <v>460</v>
+      </c>
+      <c r="C58">
+        <v>43.627676350104089</v>
+      </c>
+      <c r="D58">
+        <v>14.784357229458395</v>
+      </c>
+      <c r="F58" t="s">
+        <v>606</v>
+      </c>
+      <c r="G58">
+        <v>43.627676350104089</v>
+      </c>
+      <c r="H58">
+        <v>14.784357229458395</v>
+      </c>
+    </row>
+    <row r="59" spans="2:8">
+      <c r="B59" t="s">
+        <v>461</v>
+      </c>
+      <c r="C59">
+        <v>43.591165258465011</v>
+      </c>
+      <c r="D59">
+        <v>15.29247015684356</v>
+      </c>
+      <c r="F59" t="s">
+        <v>607</v>
+      </c>
+      <c r="G59">
+        <v>43.591165258465011</v>
+      </c>
+      <c r="H59">
+        <v>15.29247015684356</v>
+      </c>
+    </row>
+    <row r="60" spans="2:8">
+      <c r="B60" t="s">
+        <v>462</v>
+      </c>
+      <c r="C60">
+        <v>43.37637801093836</v>
+      </c>
+      <c r="D60">
+        <v>15.968965318614128</v>
+      </c>
+      <c r="F60" t="s">
+        <v>608</v>
+      </c>
+      <c r="G60">
+        <v>43.37637801093836</v>
+      </c>
+      <c r="H60">
+        <v>15.968965318614128</v>
+      </c>
+    </row>
+    <row r="61" spans="2:8">
+      <c r="B61" t="s">
+        <v>463</v>
+      </c>
+      <c r="C61">
+        <v>42.971078542317287</v>
+      </c>
+      <c r="D61">
+        <v>16.007105690349647</v>
+      </c>
+      <c r="F61" t="s">
+        <v>609</v>
+      </c>
+      <c r="G61">
+        <v>42.971078542317287</v>
+      </c>
+      <c r="H61">
+        <v>16.007105690349647</v>
+      </c>
+    </row>
+    <row r="62" spans="2:8">
+      <c r="B62" t="s">
+        <v>464</v>
+      </c>
+      <c r="C62">
+        <v>42.966936368464943</v>
+      </c>
+      <c r="D62">
+        <v>16.584950810525882</v>
+      </c>
+      <c r="F62" t="s">
+        <v>610</v>
+      </c>
+      <c r="G62">
+        <v>42.966936368464943</v>
+      </c>
+      <c r="H62">
+        <v>16.584950810525882</v>
+      </c>
+    </row>
+    <row r="63" spans="2:8">
+      <c r="B63" t="s">
+        <v>465</v>
+      </c>
+      <c r="C63">
+        <v>43.003374766865043</v>
+      </c>
+      <c r="D63">
+        <v>15.32111484630331</v>
+      </c>
+      <c r="F63" t="s">
+        <v>611</v>
+      </c>
+      <c r="G63">
+        <v>43.003374766865043</v>
+      </c>
+      <c r="H63">
+        <v>15.32111484630331</v>
+      </c>
+    </row>
+    <row r="64" spans="2:8">
+      <c r="B64" t="s">
+        <v>466</v>
+      </c>
+      <c r="C64">
+        <v>42.586922315856633</v>
+      </c>
+      <c r="D64">
+        <v>15.939538105161402</v>
+      </c>
+      <c r="F64" t="s">
+        <v>612</v>
+      </c>
+      <c r="G64">
+        <v>42.586922315856633</v>
+      </c>
+      <c r="H64">
+        <v>15.939538105161402</v>
+      </c>
+    </row>
+    <row r="65" spans="2:8">
+      <c r="B65" t="s">
+        <v>412</v>
+      </c>
+      <c r="C65">
+        <v>45.653333330000002</v>
+      </c>
+      <c r="D65">
+        <v>16.463333330000001</v>
+      </c>
+      <c r="F65" t="s">
+        <v>613</v>
+      </c>
+      <c r="G65">
+        <v>45.288705409625472</v>
+      </c>
+      <c r="H65">
+        <v>18.420983798347297</v>
+      </c>
+    </row>
+    <row r="66" spans="2:8">
+      <c r="B66" t="s">
+        <v>413</v>
+      </c>
+      <c r="C66">
+        <v>45.653333330000002</v>
+      </c>
+      <c r="D66">
+        <v>16.463611109999999</v>
+      </c>
+      <c r="F66" t="s">
+        <v>614</v>
+      </c>
+      <c r="G66">
+        <v>43.756388757532321</v>
+      </c>
+      <c r="H66">
+        <v>15.903205816155046</v>
+      </c>
+    </row>
+    <row r="67" spans="2:8">
+      <c r="B67" t="s">
+        <v>414</v>
+      </c>
+      <c r="C67">
+        <v>45.653333330000002</v>
+      </c>
+      <c r="D67">
+        <v>16.46388889</v>
+      </c>
+      <c r="F67" t="s">
+        <v>615</v>
+      </c>
+      <c r="G67">
+        <v>44.207396025652962</v>
+      </c>
+      <c r="H67">
+        <v>15.754697507990151</v>
+      </c>
+    </row>
+    <row r="68" spans="2:8">
+      <c r="B68" t="s">
+        <v>415</v>
+      </c>
+      <c r="C68">
+        <v>45.884999999999998</v>
+      </c>
+      <c r="D68">
+        <v>17.606666669999999</v>
+      </c>
+      <c r="F68" t="s">
+        <v>616</v>
+      </c>
+      <c r="G68">
+        <v>45.452492401724257</v>
+      </c>
+      <c r="H68">
+        <v>16.41378481811703</v>
+      </c>
+    </row>
+    <row r="69" spans="2:8">
+      <c r="B69" t="s">
+        <v>416</v>
+      </c>
+      <c r="C69">
+        <v>45.508888890000001</v>
+      </c>
+      <c r="D69">
+        <v>18.68</v>
+      </c>
+      <c r="F69" t="s">
+        <v>617</v>
+      </c>
+      <c r="G69">
+        <v>45.137590945224346</v>
+      </c>
+      <c r="H69">
+        <v>14.166639022574504</v>
+      </c>
+    </row>
+    <row r="70" spans="2:8">
+      <c r="B70" t="s">
+        <v>417</v>
+      </c>
+      <c r="C70">
+        <v>43.53</v>
+      </c>
+      <c r="D70">
+        <v>15.198888889999999</v>
+      </c>
+      <c r="F70" t="s">
+        <v>618</v>
+      </c>
+      <c r="G70">
+        <v>44.993014847588817</v>
+      </c>
+      <c r="H70">
+        <v>15.105276725972995</v>
+      </c>
+    </row>
+    <row r="71" spans="2:8">
+      <c r="B71" t="s">
+        <v>418</v>
+      </c>
+      <c r="C71">
+        <v>45.68305556</v>
+      </c>
+      <c r="D71">
+        <v>16.407222220000001</v>
+      </c>
+      <c r="F71" t="s">
+        <v>619</v>
+      </c>
+      <c r="G71">
+        <v>43.600259258254958</v>
+      </c>
+      <c r="H71">
+        <v>16.500996377679218</v>
+      </c>
+    </row>
+    <row r="72" spans="2:8">
+      <c r="B72" t="s">
+        <v>419</v>
+      </c>
+      <c r="C72">
+        <v>46.1875</v>
+      </c>
+      <c r="D72">
+        <v>16.97361111</v>
+      </c>
+      <c r="F72" t="s">
+        <v>620</v>
+      </c>
+      <c r="G72">
+        <v>43.60043328704915</v>
+      </c>
+      <c r="H72">
+        <v>16.501279071484671</v>
+      </c>
+    </row>
+    <row r="73" spans="2:8">
+      <c r="B73" t="s">
+        <v>420</v>
+      </c>
+      <c r="C73">
+        <v>46.108055559999997</v>
+      </c>
+      <c r="D73">
+        <v>17.106111110000001</v>
+      </c>
+      <c r="F73" t="s">
+        <v>621</v>
+      </c>
+      <c r="G73">
+        <v>45.316184595349739</v>
+      </c>
+      <c r="H73">
+        <v>14.563904567364178</v>
+      </c>
+    </row>
+    <row r="74" spans="2:8">
+      <c r="B74" t="s">
+        <v>421</v>
+      </c>
+      <c r="C74">
+        <v>45.701944439999998</v>
+      </c>
+      <c r="D74">
+        <v>18.098333329999999</v>
+      </c>
+      <c r="F74" t="s">
+        <v>622</v>
+      </c>
+      <c r="G74">
+        <v>45.31636366839107</v>
+      </c>
+      <c r="H74">
+        <v>14.564190054501609</v>
+      </c>
+    </row>
+    <row r="75" spans="2:8">
+      <c r="B75" t="s">
+        <v>422</v>
+      </c>
+      <c r="C75">
+        <v>44.333888889999997</v>
+      </c>
+      <c r="D75">
+        <v>13.498055559999999</v>
+      </c>
+      <c r="F75" t="s">
+        <v>623</v>
+      </c>
+      <c r="G75">
+        <v>45.681428265735541</v>
+      </c>
+      <c r="H75">
+        <v>15.869401606746242</v>
+      </c>
+    </row>
+    <row r="76" spans="2:8">
+      <c r="B76" t="s">
+        <v>423</v>
+      </c>
+      <c r="C76">
+        <v>44.410277780000001</v>
+      </c>
+      <c r="D76">
+        <v>13.531388890000001</v>
+      </c>
+      <c r="F76" t="s">
+        <v>624</v>
+      </c>
+      <c r="G76">
+        <v>45.667427381860662</v>
+      </c>
+      <c r="H76">
+        <v>16.111889141850742</v>
+      </c>
+    </row>
+    <row r="77" spans="2:8">
+      <c r="B77" t="s">
+        <v>424</v>
+      </c>
+      <c r="C77">
+        <v>43.518611110000002</v>
+      </c>
+      <c r="D77">
+        <v>15.142777779999999</v>
+      </c>
+      <c r="F77" t="s">
+        <v>625</v>
+      </c>
+      <c r="G77">
+        <v>45.876171942571233</v>
+      </c>
+      <c r="H77">
+        <v>16.162877551551272</v>
+      </c>
+    </row>
+    <row r="78" spans="2:8">
+      <c r="B78" t="s">
+        <v>425</v>
+      </c>
+      <c r="C78">
+        <v>43.538888890000003</v>
+      </c>
+      <c r="D78">
+        <v>15.36444444</v>
+      </c>
+      <c r="F78" t="s">
+        <v>626</v>
+      </c>
+      <c r="G78">
+        <v>45.473186839980002</v>
+      </c>
+      <c r="H78">
+        <v>18.663329039744493</v>
+      </c>
+    </row>
+    <row r="79" spans="2:8">
+      <c r="B79" t="s">
+        <v>426</v>
+      </c>
+      <c r="C79">
+        <v>43.5</v>
+      </c>
+      <c r="D79">
+        <v>15.142777779999999</v>
+      </c>
+      <c r="F79" t="s">
+        <v>627</v>
+      </c>
+      <c r="G79">
+        <v>45.448081289056574</v>
+      </c>
+      <c r="H79">
+        <v>16.913620388699012</v>
+      </c>
+    </row>
+    <row r="80" spans="2:8">
+      <c r="B80" t="s">
+        <v>427</v>
+      </c>
+      <c r="C80">
+        <v>43.523299999999999</v>
+      </c>
+      <c r="D80">
+        <v>15.36444444</v>
+      </c>
+      <c r="F80" t="s">
+        <v>628</v>
+      </c>
+      <c r="G80">
+        <v>45.653333330000002</v>
+      </c>
+      <c r="H80">
+        <v>16.463333330000001</v>
+      </c>
+    </row>
+    <row r="81" spans="6:8">
+      <c r="F81" t="s">
+        <v>629</v>
+      </c>
+      <c r="G81">
+        <v>45.653333330000002</v>
+      </c>
+      <c r="H81">
+        <v>16.463611109999999</v>
+      </c>
+    </row>
+    <row r="82" spans="6:8">
+      <c r="F82" t="s">
+        <v>630</v>
+      </c>
+      <c r="G82">
+        <v>45.653333330000002</v>
+      </c>
+      <c r="H82">
+        <v>16.46388889</v>
+      </c>
+    </row>
+    <row r="83" spans="6:8">
+      <c r="F83" t="s">
+        <v>631</v>
+      </c>
+      <c r="G83">
+        <v>45.884999999999998</v>
+      </c>
+      <c r="H83">
+        <v>17.606666669999999</v>
+      </c>
+    </row>
+    <row r="84" spans="6:8">
+      <c r="F84" t="s">
+        <v>632</v>
+      </c>
+      <c r="G84">
+        <v>45.508888890000001</v>
+      </c>
+      <c r="H84">
+        <v>18.68</v>
+      </c>
+    </row>
+    <row r="85" spans="6:8">
+      <c r="F85" t="s">
+        <v>633</v>
+      </c>
+      <c r="G85">
+        <v>43.53</v>
+      </c>
+      <c r="H85">
+        <v>15.198888889999999</v>
+      </c>
+    </row>
+    <row r="86" spans="6:8">
+      <c r="F86" t="s">
+        <v>634</v>
+      </c>
+      <c r="G86">
+        <v>45.68305556</v>
+      </c>
+      <c r="H86">
+        <v>16.407222220000001</v>
+      </c>
+    </row>
+    <row r="87" spans="6:8">
+      <c r="F87" t="s">
+        <v>635</v>
+      </c>
+      <c r="G87">
+        <v>46.1875</v>
+      </c>
+      <c r="H87">
+        <v>16.97361111</v>
+      </c>
+    </row>
+    <row r="88" spans="6:8">
+      <c r="F88" t="s">
+        <v>636</v>
+      </c>
+      <c r="G88">
+        <v>46.108055559999997</v>
+      </c>
+      <c r="H88">
+        <v>17.106111110000001</v>
+      </c>
+    </row>
+    <row r="89" spans="6:8">
+      <c r="F89" t="s">
+        <v>637</v>
+      </c>
+      <c r="G89">
+        <v>45.701944439999998</v>
+      </c>
+      <c r="H89">
+        <v>18.098333329999999</v>
+      </c>
+    </row>
+    <row r="90" spans="6:8">
+      <c r="F90" t="s">
+        <v>638</v>
+      </c>
+      <c r="G90">
+        <v>44.333888889999997</v>
+      </c>
+      <c r="H90">
+        <v>13.498055559999999</v>
+      </c>
+    </row>
+    <row r="91" spans="6:8">
+      <c r="F91" t="s">
+        <v>639</v>
+      </c>
+      <c r="G91">
+        <v>44.410277780000001</v>
+      </c>
+      <c r="H91">
+        <v>13.531388890000001</v>
+      </c>
+    </row>
+    <row r="92" spans="6:8">
+      <c r="F92" t="s">
+        <v>640</v>
+      </c>
+      <c r="G92">
+        <v>43.518611110000002</v>
+      </c>
+      <c r="H92">
+        <v>15.142777779999999</v>
+      </c>
+    </row>
+    <row r="93" spans="6:8">
+      <c r="F93" t="s">
+        <v>641</v>
+      </c>
+      <c r="G93">
+        <v>43.538888890000003</v>
+      </c>
+      <c r="H93">
+        <v>15.36444444</v>
+      </c>
+    </row>
+    <row r="94" spans="6:8">
+      <c r="F94" t="s">
+        <v>642</v>
+      </c>
+      <c r="G94">
+        <v>43.5</v>
+      </c>
+      <c r="H94">
+        <v>15.142777779999999</v>
+      </c>
+    </row>
+    <row r="95" spans="6:8">
+      <c r="F95" t="s">
+        <v>643</v>
+      </c>
+      <c r="G95">
+        <v>43.523299999999999</v>
+      </c>
+      <c r="H95">
+        <v>15.36444444</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated HRV_grids_kan10 model - 2026-08-27 13:18
</commit_message>
<xml_diff>
--- a/VerveStacks_HRV_grids_kan10/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_HRV_grids_kan10/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_HRV_grids_kan10\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{06CEF92E-74AF-48B8-8439-E10CEA7165C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{302305F1-9339-4876-9B57-A01152DEEFDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="8" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2943,7 +2943,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42CFE670-67E0-4416-855C-F02BC7EDF6DC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3DFD726-B48B-44CA-91F2-B33F376550C1}">
   <dimension ref="B9:L95"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -27032,7 +27032,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D236420-6A83-4679-9382-901650BE12E7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FD75C13-62CB-4B29-B852-922115793780}">
   <dimension ref="B9:H95"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>